<commit_message>
* * 【2025/06/17 定例会】
１．各自の立替分の精算
　　＊メイン口座の残額は、先月より54万円増えたが、偶数月に振込まれる下記保険金収入68万円によるものである。
　　 		国民厚生年金　		45
 			パナ年金　　　  	12
 			全労済個人年金  	 2
 			ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 	 9
　　　　従って、今月のメイン口座の支出は14万円前後ということになる？
　　＊共通口座の残額は、先月より30万円減ったが、金華山と網代の旅行イベントが２つあったためである。。
　　　　　(1)保険料
　　　　　(2)生活費
　　　　　　　　・小遣い振込			 	 7
　　　　　　　　・現金立替分				15			カイロとCPAPによる7万円出費を含む
　　　　　　　　・その他カード引落分		 ?
　　　　　(3)イベント費
　　　　　　　　・金華山					10?			前払い金を除く
　　　　　　　　・網代						 1			左記は土産代で、そのほ他の費用は精算中。

２．収支の確認
　　＊メイン口座は想定通り。
　　＊共通口座では保険料と生活費を合わせて毎月33万円（＝400/12）を見込んでいるのに対し、
　　　30万円の減少になっているのは金額的にはあっている。
　　　但し、これはベント費用が前払いされていたり、精算中で未払いになっているためであり、
　　　月毎の集計では費用の内訳と対応させるがが難しい。

３．メイン口座と共通口座のバランス確認
　　＊特になし

４．計画（ライフプラン.xlsx）の修正
　　＊特になし
</commit_message>
<xml_diff>
--- a/ライフプラン_猪飼.xlsx
+++ b/ライフプラン_猪飼.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC_USER\Documents\LocalLifeplanRepo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D80DBF-71B6-44B5-95AE-A14045D76F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69ED5398-DEAC-40DB-A7A6-FDDD395D3F6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{934FA03D-99BD-49E0-BFEC-291BD79F4879}"/>
   </bookViews>
@@ -72,7 +72,7 @@
           <t>マンション片付け
 キッチン（食洗器＋ガス台＋レンジ＋網戸）取替
 トイレ修理
-内壁除去</t>
+リビング内壁除去　＋　書斎クローゼット除去</t>
         </r>
       </text>
     </comment>
@@ -737,7 +737,53 @@
         </r>
       </text>
     </comment>
+    <comment ref="G113" authorId="0" shapeId="0" xr:uid="{3867A11D-F368-47C4-B52D-35EE01EC474A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>kaz
+ 国民厚生年金　　+45
+ パナ年金　　　  +12
+ 全労済個人年金  + 2　
+ ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 + 9
+nao</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="F126" authorId="0" shapeId="0" xr:uid="{9D0EDA07-5D89-456F-A52C-3AAD29C57E72}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>PC_USER:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E131" authorId="0" shapeId="0" xr:uid="{D3A0D358-7411-4045-8E31-BB4827CBD402}">
       <text>
         <r>
           <rPr>
@@ -809,18 +855,8 @@
             <family val="3"/>
             <charset val="128"/>
           </rPr>
-          <t>PC_USER:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="MS P ゴシック"/>
-            <family val="3"/>
-            <charset val="128"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
+          <t>kazへ返済 -12 (ｶｲﾛ：6、CPAP：1、中山会：１。ﾋﾞｭｰ：1。医療費他)
+naoへ返済 -3（網代0.5、出雲＆瀬戸0.4、牛乳交通費食品等2）</t>
         </r>
       </text>
     </comment>
@@ -3709,6 +3745,109 @@
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" textRotation="255"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="42" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="1" applyBorder="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" textRotation="255"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" textRotation="255"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -3718,10 +3857,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" textRotation="255"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" textRotation="255"/>
@@ -3775,105 +3910,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" textRotation="255"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="42" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" textRotation="255"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="1" applyBorder="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5571,7 +5607,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>1080</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -9023,7 +9059,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>733</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -12474,7 +12510,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>1813</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -16410,12 +16446,12 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="99" t="s">
+      <c r="B1" s="128" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="101"/>
+      <c r="C1" s="129"/>
+      <c r="D1" s="129"/>
+      <c r="E1" s="130"/>
       <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
@@ -16516,13 +16552,13 @@
       <c r="AM1" s="4"/>
     </row>
     <row r="2" spans="1:39" ht="18.75" customHeight="1">
-      <c r="A2" s="102" t="s">
+      <c r="A2" s="99" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="105" t="s">
+      <c r="B2" s="133" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="112"/>
+      <c r="C2" s="140"/>
       <c r="D2" s="6" t="s">
         <v>5</v>
       </c>
@@ -16607,9 +16643,9 @@
       <c r="AM2" s="4"/>
     </row>
     <row r="3" spans="1:39" ht="19.5" thickBot="1">
-      <c r="A3" s="103"/>
-      <c r="B3" s="106"/>
-      <c r="C3" s="113"/>
+      <c r="A3" s="131"/>
+      <c r="B3" s="134"/>
+      <c r="C3" s="141"/>
       <c r="D3" s="9" t="s">
         <v>7</v>
       </c>
@@ -16710,11 +16746,11 @@
       <c r="AM3" s="4"/>
     </row>
     <row r="4" spans="1:39">
-      <c r="A4" s="103"/>
-      <c r="B4" s="105" t="s">
+      <c r="A4" s="131"/>
+      <c r="B4" s="133" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="114"/>
+      <c r="C4" s="142"/>
       <c r="D4" s="12" t="s">
         <v>10</v>
       </c>
@@ -16759,9 +16795,9 @@
       <c r="AM4" s="4"/>
     </row>
     <row r="5" spans="1:39">
-      <c r="A5" s="103"/>
-      <c r="B5" s="107"/>
-      <c r="C5" s="115"/>
+      <c r="A5" s="131"/>
+      <c r="B5" s="135"/>
+      <c r="C5" s="143"/>
       <c r="D5" s="15" t="s">
         <v>12</v>
       </c>
@@ -16806,9 +16842,9 @@
       <c r="AM5" s="4"/>
     </row>
     <row r="6" spans="1:39">
-      <c r="A6" s="103"/>
-      <c r="B6" s="107"/>
-      <c r="C6" s="115"/>
+      <c r="A6" s="131"/>
+      <c r="B6" s="135"/>
+      <c r="C6" s="143"/>
       <c r="D6" s="15"/>
       <c r="E6" s="16"/>
       <c r="F6" s="17"/>
@@ -16847,9 +16883,9 @@
       <c r="AM6" s="4"/>
     </row>
     <row r="7" spans="1:39">
-      <c r="A7" s="103"/>
-      <c r="B7" s="107"/>
-      <c r="C7" s="115"/>
+      <c r="A7" s="131"/>
+      <c r="B7" s="135"/>
+      <c r="C7" s="143"/>
       <c r="D7" s="15"/>
       <c r="E7" s="16"/>
       <c r="F7" s="17"/>
@@ -16888,9 +16924,9 @@
       <c r="AM7" s="4"/>
     </row>
     <row r="8" spans="1:39">
-      <c r="A8" s="103"/>
-      <c r="B8" s="108"/>
-      <c r="C8" s="116"/>
+      <c r="A8" s="131"/>
+      <c r="B8" s="136"/>
+      <c r="C8" s="144"/>
       <c r="D8" s="15"/>
       <c r="E8" s="16"/>
       <c r="F8" s="17"/>
@@ -16929,12 +16965,12 @@
       <c r="AM8" s="4"/>
     </row>
     <row r="9" spans="1:39" ht="19.5" thickBot="1">
-      <c r="A9" s="103"/>
-      <c r="B9" s="109" t="s">
+      <c r="A9" s="131"/>
+      <c r="B9" s="137" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="110"/>
-      <c r="D9" s="111"/>
+      <c r="C9" s="138"/>
+      <c r="D9" s="139"/>
       <c r="E9" s="18" t="s">
         <v>15</v>
       </c>
@@ -17070,11 +17106,11 @@
       <c r="AM9" s="4"/>
     </row>
     <row r="10" spans="1:39">
-      <c r="A10" s="103"/>
-      <c r="B10" s="105" t="s">
+      <c r="A10" s="131"/>
+      <c r="B10" s="133" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="114"/>
+      <c r="C10" s="142"/>
       <c r="D10" s="15" t="s">
         <v>17</v>
       </c>
@@ -17173,9 +17209,9 @@
       <c r="AM10" s="4"/>
     </row>
     <row r="11" spans="1:39">
-      <c r="A11" s="103"/>
-      <c r="B11" s="107"/>
-      <c r="C11" s="115"/>
+      <c r="A11" s="131"/>
+      <c r="B11" s="135"/>
+      <c r="C11" s="143"/>
       <c r="D11" s="15" t="s">
         <v>19</v>
       </c>
@@ -17225,9 +17261,9 @@
       <c r="AM11" s="4"/>
     </row>
     <row r="12" spans="1:39">
-      <c r="A12" s="103"/>
-      <c r="B12" s="107"/>
-      <c r="C12" s="115"/>
+      <c r="A12" s="131"/>
+      <c r="B12" s="135"/>
+      <c r="C12" s="143"/>
       <c r="D12" s="15" t="s">
         <v>21</v>
       </c>
@@ -17299,9 +17335,9 @@
       <c r="AM12" s="4"/>
     </row>
     <row r="13" spans="1:39">
-      <c r="A13" s="103"/>
-      <c r="B13" s="107"/>
-      <c r="C13" s="115"/>
+      <c r="A13" s="131"/>
+      <c r="B13" s="135"/>
+      <c r="C13" s="143"/>
       <c r="D13" s="15" t="s">
         <v>22</v>
       </c>
@@ -17350,9 +17386,9 @@
       <c r="AM13" s="4"/>
     </row>
     <row r="14" spans="1:39">
-      <c r="A14" s="103"/>
-      <c r="B14" s="108"/>
-      <c r="C14" s="116"/>
+      <c r="A14" s="131"/>
+      <c r="B14" s="136"/>
+      <c r="C14" s="144"/>
       <c r="D14" s="15"/>
       <c r="E14" s="16"/>
       <c r="F14" s="23"/>
@@ -17391,12 +17427,12 @@
       <c r="AM14" s="4"/>
     </row>
     <row r="15" spans="1:39" ht="19.5" thickBot="1">
-      <c r="A15" s="104"/>
-      <c r="B15" s="109" t="s">
+      <c r="A15" s="132"/>
+      <c r="B15" s="137" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="110"/>
-      <c r="D15" s="111"/>
+      <c r="C15" s="138"/>
+      <c r="D15" s="139"/>
       <c r="E15" s="18" t="s">
         <v>25</v>
       </c>
@@ -17532,16 +17568,16 @@
       <c r="AM15" s="4"/>
     </row>
     <row r="16" spans="1:39">
-      <c r="A16" s="102" t="s">
+      <c r="A16" s="99" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="136" t="s">
+      <c r="B16" s="126" t="s">
         <v>132</v>
       </c>
       <c r="C16" s="118" t="s">
         <v>108</v>
       </c>
-      <c r="D16" s="120" t="s">
+      <c r="D16" s="119" t="s">
         <v>112</v>
       </c>
       <c r="E16" s="16" t="s">
@@ -17623,10 +17659,10 @@
       <c r="AM16" s="4"/>
     </row>
     <row r="17" spans="1:39">
-      <c r="A17" s="138"/>
-      <c r="B17" s="134"/>
-      <c r="C17" s="119"/>
-      <c r="D17" s="119"/>
+      <c r="A17" s="100"/>
+      <c r="B17" s="124"/>
+      <c r="C17" s="107"/>
+      <c r="D17" s="107"/>
       <c r="E17" s="16" t="s">
         <v>30</v>
       </c>
@@ -17712,12 +17748,12 @@
       <c r="AM17" s="4"/>
     </row>
     <row r="18" spans="1:39">
-      <c r="A18" s="138"/>
-      <c r="B18" s="134"/>
-      <c r="C18" s="121" t="s">
+      <c r="A18" s="100"/>
+      <c r="B18" s="124"/>
+      <c r="C18" s="110" t="s">
         <v>109</v>
       </c>
-      <c r="D18" s="123" t="s">
+      <c r="D18" s="111" t="s">
         <v>114</v>
       </c>
       <c r="E18" s="13" t="s">
@@ -17799,10 +17835,10 @@
       <c r="AM18" s="27"/>
     </row>
     <row r="19" spans="1:39">
-      <c r="A19" s="138"/>
-      <c r="B19" s="134"/>
-      <c r="C19" s="122"/>
-      <c r="D19" s="122"/>
+      <c r="A19" s="100"/>
+      <c r="B19" s="124"/>
+      <c r="C19" s="112"/>
+      <c r="D19" s="112"/>
       <c r="E19" s="16" t="s">
         <v>28</v>
       </c>
@@ -17870,10 +17906,10 @@
       <c r="AM19" s="27"/>
     </row>
     <row r="20" spans="1:39">
-      <c r="A20" s="138"/>
-      <c r="B20" s="134"/>
-      <c r="C20" s="122"/>
-      <c r="D20" s="119"/>
+      <c r="A20" s="100"/>
+      <c r="B20" s="124"/>
+      <c r="C20" s="112"/>
+      <c r="D20" s="107"/>
       <c r="E20" s="16" t="s">
         <v>29</v>
       </c>
@@ -17923,9 +17959,9 @@
       <c r="AM20" s="27"/>
     </row>
     <row r="21" spans="1:39">
-      <c r="A21" s="138"/>
-      <c r="B21" s="134"/>
-      <c r="C21" s="119"/>
+      <c r="A21" s="100"/>
+      <c r="B21" s="124"/>
+      <c r="C21" s="107"/>
       <c r="D21" s="57" t="s">
         <v>115</v>
       </c>
@@ -17976,9 +18012,9 @@
       <c r="AM21" s="27"/>
     </row>
     <row r="22" spans="1:39">
-      <c r="A22" s="138"/>
-      <c r="B22" s="134"/>
-      <c r="C22" s="121" t="s">
+      <c r="A22" s="100"/>
+      <c r="B22" s="124"/>
+      <c r="C22" s="110" t="s">
         <v>110</v>
       </c>
       <c r="D22" s="57" t="s">
@@ -18023,9 +18059,9 @@
       <c r="AM22" s="27"/>
     </row>
     <row r="23" spans="1:39">
-      <c r="A23" s="138"/>
-      <c r="B23" s="134"/>
-      <c r="C23" s="119"/>
+      <c r="A23" s="100"/>
+      <c r="B23" s="124"/>
+      <c r="C23" s="107"/>
       <c r="D23" s="57" t="s">
         <v>117</v>
       </c>
@@ -18068,12 +18104,12 @@
       <c r="AM23" s="27"/>
     </row>
     <row r="24" spans="1:39">
-      <c r="A24" s="138"/>
-      <c r="B24" s="134"/>
-      <c r="C24" s="121" t="s">
+      <c r="A24" s="100"/>
+      <c r="B24" s="124"/>
+      <c r="C24" s="110" t="s">
         <v>111</v>
       </c>
-      <c r="D24" s="123" t="s">
+      <c r="D24" s="111" t="s">
         <v>118</v>
       </c>
       <c r="E24" s="16" t="s">
@@ -18155,10 +18191,10 @@
       <c r="AM24" s="27"/>
     </row>
     <row r="25" spans="1:39">
-      <c r="A25" s="138"/>
-      <c r="B25" s="134"/>
-      <c r="C25" s="122"/>
-      <c r="D25" s="122"/>
+      <c r="A25" s="100"/>
+      <c r="B25" s="124"/>
+      <c r="C25" s="112"/>
+      <c r="D25" s="112"/>
       <c r="E25" s="16" t="s">
         <v>33</v>
       </c>
@@ -18250,10 +18286,10 @@
       <c r="AM25" s="27"/>
     </row>
     <row r="26" spans="1:39">
-      <c r="A26" s="138"/>
-      <c r="B26" s="134"/>
-      <c r="C26" s="122"/>
-      <c r="D26" s="122"/>
+      <c r="A26" s="100"/>
+      <c r="B26" s="124"/>
+      <c r="C26" s="112"/>
+      <c r="D26" s="112"/>
       <c r="E26" s="16" t="s">
         <v>34</v>
       </c>
@@ -18295,10 +18331,10 @@
       <c r="AM26" s="27"/>
     </row>
     <row r="27" spans="1:39">
-      <c r="A27" s="138"/>
-      <c r="B27" s="134"/>
-      <c r="C27" s="122"/>
-      <c r="D27" s="122"/>
+      <c r="A27" s="100"/>
+      <c r="B27" s="124"/>
+      <c r="C27" s="112"/>
+      <c r="D27" s="112"/>
       <c r="E27" s="29" t="s">
         <v>35</v>
       </c>
@@ -18340,10 +18376,10 @@
       <c r="AM27" s="27"/>
     </row>
     <row r="28" spans="1:39">
-      <c r="A28" s="138"/>
-      <c r="B28" s="134"/>
-      <c r="C28" s="122"/>
-      <c r="D28" s="122"/>
+      <c r="A28" s="100"/>
+      <c r="B28" s="124"/>
+      <c r="C28" s="112"/>
+      <c r="D28" s="112"/>
       <c r="E28" s="16" t="s">
         <v>36</v>
       </c>
@@ -18403,10 +18439,10 @@
       <c r="AM28" s="27"/>
     </row>
     <row r="29" spans="1:39">
-      <c r="A29" s="138"/>
-      <c r="B29" s="134"/>
-      <c r="C29" s="122"/>
-      <c r="D29" s="119"/>
+      <c r="A29" s="100"/>
+      <c r="B29" s="124"/>
+      <c r="C29" s="112"/>
+      <c r="D29" s="107"/>
       <c r="E29" s="86" t="s">
         <v>120</v>
       </c>
@@ -18448,9 +18484,9 @@
       <c r="AM29" s="27"/>
     </row>
     <row r="30" spans="1:39">
-      <c r="A30" s="138"/>
-      <c r="B30" s="134"/>
-      <c r="C30" s="122"/>
+      <c r="A30" s="100"/>
+      <c r="B30" s="124"/>
+      <c r="C30" s="112"/>
       <c r="D30" s="57" t="s">
         <v>122</v>
       </c>
@@ -18493,9 +18529,9 @@
       <c r="AM30" s="27"/>
     </row>
     <row r="31" spans="1:39">
-      <c r="A31" s="138"/>
-      <c r="B31" s="135"/>
-      <c r="C31" s="119"/>
+      <c r="A31" s="100"/>
+      <c r="B31" s="125"/>
+      <c r="C31" s="107"/>
       <c r="D31" s="57" t="s">
         <v>123</v>
       </c>
@@ -18538,11 +18574,11 @@
       <c r="AM31" s="27"/>
     </row>
     <row r="32" spans="1:39">
-      <c r="A32" s="138"/>
-      <c r="B32" s="143" t="s">
+      <c r="A32" s="100"/>
+      <c r="B32" s="115" t="s">
         <v>131</v>
       </c>
-      <c r="C32" s="124"/>
+      <c r="C32" s="108"/>
       <c r="D32" s="17" t="s">
         <v>128</v>
       </c>
@@ -18641,9 +18677,9 @@
       <c r="AM32" s="27"/>
     </row>
     <row r="33" spans="1:39">
-      <c r="A33" s="138"/>
-      <c r="B33" s="144"/>
-      <c r="C33" s="126"/>
+      <c r="A33" s="100"/>
+      <c r="B33" s="116"/>
+      <c r="C33" s="105"/>
       <c r="D33" s="17" t="s">
         <v>129</v>
       </c>
@@ -18718,12 +18754,12 @@
       <c r="AM33" s="27"/>
     </row>
     <row r="34" spans="1:39">
-      <c r="A34" s="138"/>
-      <c r="B34" s="127" t="s">
+      <c r="A34" s="100"/>
+      <c r="B34" s="102" t="s">
         <v>9</v>
       </c>
-      <c r="C34" s="130"/>
-      <c r="D34" s="140"/>
+      <c r="C34" s="104"/>
+      <c r="D34" s="106"/>
       <c r="E34" s="34" t="str">
         <f t="shared" ref="E34:AK34" si="2">E4</f>
         <v>新潟実家の売却益　（妙子と折半）</v>
@@ -18860,10 +18896,10 @@
       <c r="AM34" s="27"/>
     </row>
     <row r="35" spans="1:39">
-      <c r="A35" s="138"/>
-      <c r="B35" s="129"/>
-      <c r="C35" s="126"/>
-      <c r="D35" s="119"/>
+      <c r="A35" s="100"/>
+      <c r="B35" s="103"/>
+      <c r="C35" s="105"/>
+      <c r="D35" s="107"/>
       <c r="E35" s="34" t="str">
         <f t="shared" ref="E35:AK35" si="3">E5</f>
         <v>横浜マンションの売却益</v>
@@ -19000,7 +19036,7 @@
       <c r="AM35" s="27"/>
     </row>
     <row r="36" spans="1:39" ht="19.5" thickBot="1">
-      <c r="A36" s="138"/>
+      <c r="A36" s="100"/>
       <c r="B36" s="35" t="s">
         <v>38</v>
       </c>
@@ -19139,8 +19175,8 @@
       <c r="AM36" s="27"/>
     </row>
     <row r="37" spans="1:39">
-      <c r="A37" s="138"/>
-      <c r="B37" s="133" t="s">
+      <c r="A37" s="100"/>
+      <c r="B37" s="123" t="s">
         <v>133</v>
       </c>
       <c r="C37" s="8" t="s">
@@ -19190,9 +19226,9 @@
       <c r="AM37" s="4"/>
     </row>
     <row r="38" spans="1:39">
-      <c r="A38" s="138"/>
-      <c r="B38" s="134"/>
-      <c r="C38" s="121" t="s">
+      <c r="A38" s="100"/>
+      <c r="B38" s="124"/>
+      <c r="C38" s="110" t="s">
         <v>109</v>
       </c>
       <c r="D38" s="57" t="s">
@@ -19237,9 +19273,9 @@
       <c r="AM38" s="4"/>
     </row>
     <row r="39" spans="1:39">
-      <c r="A39" s="138"/>
-      <c r="B39" s="134"/>
-      <c r="C39" s="119"/>
+      <c r="A39" s="100"/>
+      <c r="B39" s="124"/>
+      <c r="C39" s="107"/>
       <c r="D39" s="57" t="s">
         <v>115</v>
       </c>
@@ -19282,9 +19318,9 @@
       <c r="AM39" s="4"/>
     </row>
     <row r="40" spans="1:39">
-      <c r="A40" s="138"/>
-      <c r="B40" s="134"/>
-      <c r="C40" s="121" t="s">
+      <c r="A40" s="100"/>
+      <c r="B40" s="124"/>
+      <c r="C40" s="110" t="s">
         <v>110</v>
       </c>
       <c r="D40" s="57" t="s">
@@ -19385,9 +19421,9 @@
       <c r="AM40" s="27"/>
     </row>
     <row r="41" spans="1:39">
-      <c r="A41" s="138"/>
-      <c r="B41" s="134"/>
-      <c r="C41" s="119"/>
+      <c r="A41" s="100"/>
+      <c r="B41" s="124"/>
+      <c r="C41" s="107"/>
       <c r="D41" s="57" t="s">
         <v>117</v>
       </c>
@@ -19430,12 +19466,12 @@
       <c r="AM41" s="4"/>
     </row>
     <row r="42" spans="1:39">
-      <c r="A42" s="138"/>
-      <c r="B42" s="134"/>
-      <c r="C42" s="121" t="s">
+      <c r="A42" s="100"/>
+      <c r="B42" s="124"/>
+      <c r="C42" s="110" t="s">
         <v>111</v>
       </c>
-      <c r="D42" s="123" t="s">
+      <c r="D42" s="111" t="s">
         <v>118</v>
       </c>
       <c r="E42" s="16" t="s">
@@ -19481,10 +19517,10 @@
       <c r="AM42" s="27"/>
     </row>
     <row r="43" spans="1:39">
-      <c r="A43" s="138"/>
-      <c r="B43" s="134"/>
-      <c r="C43" s="122"/>
-      <c r="D43" s="122"/>
+      <c r="A43" s="100"/>
+      <c r="B43" s="124"/>
+      <c r="C43" s="112"/>
+      <c r="D43" s="112"/>
       <c r="E43" s="16" t="s">
         <v>49</v>
       </c>
@@ -19564,10 +19600,10 @@
       <c r="AM43" s="27"/>
     </row>
     <row r="44" spans="1:39">
-      <c r="A44" s="138"/>
-      <c r="B44" s="134"/>
-      <c r="C44" s="122"/>
-      <c r="D44" s="122"/>
+      <c r="A44" s="100"/>
+      <c r="B44" s="124"/>
+      <c r="C44" s="112"/>
+      <c r="D44" s="112"/>
       <c r="E44" s="16" t="s">
         <v>50</v>
       </c>
@@ -19639,10 +19675,10 @@
       <c r="AM44" s="27"/>
     </row>
     <row r="45" spans="1:39">
-      <c r="A45" s="138"/>
-      <c r="B45" s="134"/>
-      <c r="C45" s="122"/>
-      <c r="D45" s="119"/>
+      <c r="A45" s="100"/>
+      <c r="B45" s="124"/>
+      <c r="C45" s="112"/>
+      <c r="D45" s="107"/>
       <c r="E45" s="86" t="s">
         <v>124</v>
       </c>
@@ -19692,9 +19728,9 @@
       <c r="AM45" s="27"/>
     </row>
     <row r="46" spans="1:39">
-      <c r="A46" s="138"/>
-      <c r="B46" s="134"/>
-      <c r="C46" s="122"/>
+      <c r="A46" s="100"/>
+      <c r="B46" s="124"/>
+      <c r="C46" s="112"/>
       <c r="D46" s="57" t="s">
         <v>122</v>
       </c>
@@ -19787,9 +19823,9 @@
       <c r="AM46" s="27"/>
     </row>
     <row r="47" spans="1:39">
-      <c r="A47" s="138"/>
-      <c r="B47" s="135"/>
-      <c r="C47" s="119"/>
+      <c r="A47" s="100"/>
+      <c r="B47" s="125"/>
+      <c r="C47" s="107"/>
       <c r="D47" s="57" t="s">
         <v>123</v>
       </c>
@@ -19832,7 +19868,7 @@
       <c r="AM47" s="4"/>
     </row>
     <row r="48" spans="1:39">
-      <c r="A48" s="138"/>
+      <c r="A48" s="100"/>
       <c r="B48" s="66" t="s">
         <v>45</v>
       </c>
@@ -19917,7 +19953,7 @@
       <c r="AM48" s="27"/>
     </row>
     <row r="49" spans="1:39">
-      <c r="A49" s="138"/>
+      <c r="A49" s="100"/>
       <c r="B49" s="66" t="s">
         <v>52</v>
       </c>
@@ -20018,7 +20054,7 @@
       <c r="AM49" s="27"/>
     </row>
     <row r="50" spans="1:39">
-      <c r="A50" s="138"/>
+      <c r="A50" s="100"/>
       <c r="B50" s="66" t="s">
         <v>54</v>
       </c>
@@ -20119,11 +20155,11 @@
       <c r="AM50" s="27"/>
     </row>
     <row r="51" spans="1:39">
-      <c r="A51" s="138"/>
-      <c r="B51" s="132" t="s">
+      <c r="A51" s="100"/>
+      <c r="B51" s="122" t="s">
         <v>125</v>
       </c>
-      <c r="C51" s="124"/>
+      <c r="C51" s="108"/>
       <c r="D51" s="15" t="s">
         <v>43</v>
       </c>
@@ -20206,9 +20242,9 @@
       <c r="AM51" s="27"/>
     </row>
     <row r="52" spans="1:39">
-      <c r="A52" s="138"/>
-      <c r="B52" s="128"/>
-      <c r="C52" s="125"/>
+      <c r="A52" s="100"/>
+      <c r="B52" s="120"/>
+      <c r="C52" s="109"/>
       <c r="D52" s="15" t="s">
         <v>39</v>
       </c>
@@ -20253,9 +20289,9 @@
       <c r="AM52" s="27"/>
     </row>
     <row r="53" spans="1:39">
-      <c r="A53" s="138"/>
-      <c r="B53" s="129"/>
-      <c r="C53" s="126"/>
+      <c r="A53" s="100"/>
+      <c r="B53" s="103"/>
+      <c r="C53" s="105"/>
       <c r="D53" s="15" t="s">
         <v>41</v>
       </c>
@@ -20354,7 +20390,7 @@
       <c r="AM53" s="27"/>
     </row>
     <row r="54" spans="1:39">
-      <c r="A54" s="138"/>
+      <c r="A54" s="100"/>
       <c r="B54" s="84" t="s">
         <v>141</v>
       </c>
@@ -20457,11 +20493,11 @@
       <c r="AM54" s="27"/>
     </row>
     <row r="55" spans="1:39">
-      <c r="A55" s="138"/>
-      <c r="B55" s="141" t="s">
+      <c r="A55" s="100"/>
+      <c r="B55" s="113" t="s">
         <v>148</v>
       </c>
-      <c r="C55" s="142"/>
+      <c r="C55" s="114"/>
       <c r="D55" s="78" t="s">
         <v>127</v>
       </c>
@@ -20584,7 +20620,7 @@
       <c r="AM55" s="27"/>
     </row>
     <row r="56" spans="1:39">
-      <c r="A56" s="138"/>
+      <c r="A56" s="100"/>
       <c r="B56" s="67" t="s">
         <v>58</v>
       </c>
@@ -20713,7 +20749,7 @@
       <c r="AM56" s="27"/>
     </row>
     <row r="57" spans="1:39">
-      <c r="A57" s="138"/>
+      <c r="A57" s="100"/>
       <c r="B57" s="67" t="s">
         <v>60</v>
       </c>
@@ -20840,7 +20876,7 @@
       <c r="AM57" s="27"/>
     </row>
     <row r="58" spans="1:39" ht="19.5" thickBot="1">
-      <c r="A58" s="139"/>
+      <c r="A58" s="101"/>
       <c r="B58" s="61" t="s">
         <v>61</v>
       </c>
@@ -20969,7 +21005,7 @@
       <c r="AM58" s="27"/>
     </row>
     <row r="59" spans="1:39" ht="18.75" customHeight="1">
-      <c r="A59" s="102" t="s">
+      <c r="A59" s="99" t="s">
         <v>62</v>
       </c>
       <c r="B59" s="81" t="s">
@@ -21103,7 +21139,7 @@
       <c r="AM59" s="27"/>
     </row>
     <row r="60" spans="1:39" ht="19.5" thickBot="1">
-      <c r="A60" s="137"/>
+      <c r="A60" s="127"/>
       <c r="B60" s="61" t="s">
         <v>38</v>
       </c>
@@ -21233,7 +21269,7 @@
       <c r="AM60" s="27"/>
     </row>
     <row r="61" spans="1:39">
-      <c r="A61" s="137"/>
+      <c r="A61" s="127"/>
       <c r="B61" s="68" t="s">
         <v>138</v>
       </c>
@@ -21284,11 +21320,11 @@
       <c r="AM61" s="27"/>
     </row>
     <row r="62" spans="1:39">
-      <c r="A62" s="137"/>
-      <c r="B62" s="131" t="s">
+      <c r="A62" s="127"/>
+      <c r="B62" s="121" t="s">
         <v>125</v>
       </c>
-      <c r="C62" s="124"/>
+      <c r="C62" s="108"/>
       <c r="D62" s="72" t="s">
         <v>64</v>
       </c>
@@ -21387,9 +21423,9 @@
       <c r="AM62" s="27"/>
     </row>
     <row r="63" spans="1:39">
-      <c r="A63" s="137"/>
-      <c r="B63" s="128"/>
-      <c r="C63" s="125"/>
+      <c r="A63" s="127"/>
+      <c r="B63" s="120"/>
+      <c r="C63" s="109"/>
       <c r="D63" s="15" t="s">
         <v>66</v>
       </c>
@@ -21488,9 +21524,9 @@
       <c r="AM63" s="27"/>
     </row>
     <row r="64" spans="1:39">
-      <c r="A64" s="137"/>
-      <c r="B64" s="128"/>
-      <c r="C64" s="125"/>
+      <c r="A64" s="127"/>
+      <c r="B64" s="120"/>
+      <c r="C64" s="109"/>
       <c r="D64" s="15" t="s">
         <v>68</v>
       </c>
@@ -21589,9 +21625,9 @@
       <c r="AM64" s="27"/>
     </row>
     <row r="65" spans="1:39">
-      <c r="A65" s="137"/>
-      <c r="B65" s="128"/>
-      <c r="C65" s="125"/>
+      <c r="A65" s="127"/>
+      <c r="B65" s="120"/>
+      <c r="C65" s="109"/>
       <c r="D65" s="15" t="s">
         <v>70</v>
       </c>
@@ -21690,9 +21726,9 @@
       <c r="AM65" s="27"/>
     </row>
     <row r="66" spans="1:39">
-      <c r="A66" s="137"/>
-      <c r="B66" s="128"/>
-      <c r="C66" s="125"/>
+      <c r="A66" s="127"/>
+      <c r="B66" s="120"/>
+      <c r="C66" s="109"/>
       <c r="D66" s="15" t="s">
         <v>54</v>
       </c>
@@ -21791,9 +21827,9 @@
       <c r="AM66" s="27"/>
     </row>
     <row r="67" spans="1:39">
-      <c r="A67" s="137"/>
-      <c r="B67" s="128"/>
-      <c r="C67" s="125"/>
+      <c r="A67" s="127"/>
+      <c r="B67" s="120"/>
+      <c r="C67" s="109"/>
       <c r="D67" s="15" t="s">
         <v>73</v>
       </c>
@@ -21892,9 +21928,9 @@
       <c r="AM67" s="27"/>
     </row>
     <row r="68" spans="1:39">
-      <c r="A68" s="137"/>
-      <c r="B68" s="128"/>
-      <c r="C68" s="125"/>
+      <c r="A68" s="127"/>
+      <c r="B68" s="120"/>
+      <c r="C68" s="109"/>
       <c r="D68" s="15" t="s">
         <v>75</v>
       </c>
@@ -21993,9 +22029,9 @@
       <c r="AM68" s="27"/>
     </row>
     <row r="69" spans="1:39">
-      <c r="A69" s="137"/>
-      <c r="B69" s="128"/>
-      <c r="C69" s="125"/>
+      <c r="A69" s="127"/>
+      <c r="B69" s="120"/>
+      <c r="C69" s="109"/>
       <c r="D69" s="15" t="s">
         <v>77</v>
       </c>
@@ -22094,9 +22130,9 @@
       <c r="AM69" s="27"/>
     </row>
     <row r="70" spans="1:39">
-      <c r="A70" s="137"/>
-      <c r="B70" s="128"/>
-      <c r="C70" s="125"/>
+      <c r="A70" s="127"/>
+      <c r="B70" s="120"/>
+      <c r="C70" s="109"/>
       <c r="D70" s="15" t="s">
         <v>79</v>
       </c>
@@ -22195,10 +22231,10 @@
       <c r="AM70" s="27"/>
     </row>
     <row r="71" spans="1:39">
-      <c r="A71" s="137"/>
-      <c r="B71" s="128"/>
-      <c r="C71" s="125"/>
-      <c r="D71" s="121" t="s">
+      <c r="A71" s="127"/>
+      <c r="B71" s="120"/>
+      <c r="C71" s="109"/>
+      <c r="D71" s="110" t="s">
         <v>82</v>
       </c>
       <c r="E71" s="16" t="s">
@@ -22300,10 +22336,10 @@
       <c r="AM71" s="27"/>
     </row>
     <row r="72" spans="1:39">
-      <c r="A72" s="137"/>
-      <c r="B72" s="129"/>
-      <c r="C72" s="126"/>
-      <c r="D72" s="119"/>
+      <c r="A72" s="127"/>
+      <c r="B72" s="103"/>
+      <c r="C72" s="105"/>
+      <c r="D72" s="107"/>
       <c r="E72" s="16" t="s">
         <v>84</v>
       </c>
@@ -22403,11 +22439,11 @@
       <c r="AM72" s="27"/>
     </row>
     <row r="73" spans="1:39">
-      <c r="A73" s="137"/>
-      <c r="B73" s="127" t="s">
+      <c r="A73" s="127"/>
+      <c r="B73" s="102" t="s">
         <v>16</v>
       </c>
-      <c r="C73" s="130"/>
+      <c r="C73" s="104"/>
       <c r="D73" s="33" t="s">
         <v>134</v>
       </c>
@@ -22537,9 +22573,9 @@
       <c r="AM73" s="27"/>
     </row>
     <row r="74" spans="1:39">
-      <c r="A74" s="137"/>
-      <c r="B74" s="128"/>
-      <c r="C74" s="125"/>
+      <c r="A74" s="127"/>
+      <c r="B74" s="120"/>
+      <c r="C74" s="109"/>
       <c r="D74" s="33" t="s">
         <v>135</v>
       </c>
@@ -22669,9 +22705,9 @@
       <c r="AM74" s="27"/>
     </row>
     <row r="75" spans="1:39">
-      <c r="A75" s="137"/>
-      <c r="B75" s="128"/>
-      <c r="C75" s="125"/>
+      <c r="A75" s="127"/>
+      <c r="B75" s="120"/>
+      <c r="C75" s="109"/>
       <c r="D75" s="33" t="s">
         <v>136</v>
       </c>
@@ -22801,9 +22837,9 @@
       <c r="AM75" s="27"/>
     </row>
     <row r="76" spans="1:39">
-      <c r="A76" s="137"/>
-      <c r="B76" s="129"/>
-      <c r="C76" s="126"/>
+      <c r="A76" s="127"/>
+      <c r="B76" s="103"/>
+      <c r="C76" s="105"/>
       <c r="D76" s="33" t="s">
         <v>137</v>
       </c>
@@ -22933,7 +22969,7 @@
       <c r="AM76" s="27"/>
     </row>
     <row r="77" spans="1:39">
-      <c r="A77" s="137"/>
+      <c r="A77" s="127"/>
       <c r="B77" s="67" t="s">
         <v>58</v>
       </c>
@@ -23063,7 +23099,7 @@
       <c r="AM77" s="27"/>
     </row>
     <row r="78" spans="1:39">
-      <c r="A78" s="137"/>
+      <c r="A78" s="127"/>
       <c r="B78" s="67" t="s">
         <v>60</v>
       </c>
@@ -23322,7 +23358,7 @@
       <c r="AM79" s="27"/>
     </row>
     <row r="80" spans="1:39">
-      <c r="A80" s="102" t="s">
+      <c r="A80" s="99" t="s">
         <v>89</v>
       </c>
       <c r="B80" s="59" t="s">
@@ -24021,9 +24057,9 @@
       <c r="F93" s="55" t="s">
         <v>98</v>
       </c>
-      <c r="G93" s="56" t="e">
+      <c r="G93" s="56">
         <f t="shared" ref="G93:AK93" si="22">G113+G133</f>
-        <v>#N/A</v>
+        <v>1813</v>
       </c>
       <c r="H93" s="57" t="e">
         <f t="shared" si="22"/>
@@ -25778,8 +25814,8 @@
       <c r="F113" s="55" t="s">
         <v>98</v>
       </c>
-      <c r="G113" s="56" t="e">
-        <v>#N/A</v>
+      <c r="G113" s="56">
+        <v>1080</v>
       </c>
       <c r="H113" s="57" t="e">
         <v>#N/A</v>
@@ -27018,8 +27054,8 @@
         <v>151</v>
       </c>
     </row>
-    <row r="129" spans="6:37" ht="19.5" thickBot="1"/>
-    <row r="130" spans="6:37" ht="19.5" thickBot="1">
+    <row r="129" spans="5:37" ht="19.5" thickBot="1"/>
+    <row r="130" spans="5:37" ht="19.5" thickBot="1">
       <c r="F130" s="92" t="s">
         <v>107</v>
       </c>
@@ -27117,7 +27153,7 @@
         <v>2055</v>
       </c>
     </row>
-    <row r="131" spans="6:37">
+    <row r="131" spans="5:37">
       <c r="F131" s="88" t="s">
         <v>96</v>
       </c>
@@ -27216,7 +27252,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="132" spans="6:37">
+    <row r="132" spans="5:37">
       <c r="F132" s="55" t="s">
         <v>97</v>
       </c>
@@ -27314,12 +27350,12 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="133" spans="6:37">
+    <row r="133" spans="5:37">
       <c r="F133" s="55" t="s">
         <v>98</v>
       </c>
-      <c r="G133" s="56" t="e">
-        <v>#N/A</v>
+      <c r="G133" s="56">
+        <v>733</v>
       </c>
       <c r="H133" s="57" t="e">
         <v>#N/A</v>
@@ -27412,7 +27448,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="134" spans="6:37">
+    <row r="134" spans="5:37">
       <c r="F134" s="55" t="s">
         <v>99</v>
       </c>
@@ -27510,7 +27546,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="135" spans="6:37">
+    <row r="135" spans="5:37">
       <c r="F135" s="55" t="s">
         <v>100</v>
       </c>
@@ -27608,7 +27644,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="136" spans="6:37">
+    <row r="136" spans="5:37">
       <c r="F136" s="55" t="s">
         <v>101</v>
       </c>
@@ -27706,7 +27742,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="137" spans="6:37">
+    <row r="137" spans="5:37">
       <c r="F137" s="55" t="s">
         <v>102</v>
       </c>
@@ -27804,7 +27840,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="138" spans="6:37">
+    <row r="138" spans="5:37">
       <c r="F138" s="55" t="s">
         <v>103</v>
       </c>
@@ -27902,7 +27938,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="139" spans="6:37">
+    <row r="139" spans="5:37">
       <c r="F139" s="89" t="s">
         <v>104</v>
       </c>
@@ -28000,7 +28036,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="140" spans="6:37">
+    <row r="140" spans="5:37">
       <c r="F140" s="89" t="s">
         <v>93</v>
       </c>
@@ -28098,7 +28134,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="141" spans="6:37">
+    <row r="141" spans="5:37">
       <c r="F141" s="55" t="s">
         <v>94</v>
       </c>
@@ -28196,7 +28232,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="142" spans="6:37" ht="19.5" thickBot="1">
+    <row r="142" spans="5:37" ht="19.5" thickBot="1">
       <c r="F142" s="97" t="s">
         <v>95</v>
       </c>
@@ -28294,7 +28330,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="143" spans="6:37">
+    <row r="143" spans="5:37">
       <c r="F143" s="59" t="s">
         <v>105</v>
       </c>
@@ -28423,7 +28459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="6:37" ht="19.5" thickBot="1">
+    <row r="144" spans="5:37" ht="19.5" thickBot="1">
       <c r="F144" s="61" t="s">
         <v>106</v>
       </c>
@@ -28554,19 +28590,16 @@
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="A16:A58"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="C62:C72"/>
-    <mergeCell ref="D71:D72"/>
-    <mergeCell ref="D24:D29"/>
-    <mergeCell ref="D42:D45"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="C42:C47"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A2:A15"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="B4:B8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:B14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C4:C8"/>
+    <mergeCell ref="C10:C14"/>
     <mergeCell ref="A80:A81"/>
     <mergeCell ref="C16:C17"/>
     <mergeCell ref="D16:D17"/>
@@ -28583,16 +28616,19 @@
     <mergeCell ref="B37:B47"/>
     <mergeCell ref="B16:B31"/>
     <mergeCell ref="A59:A79"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="A2:A15"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B4:B8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:B14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C4:C8"/>
-    <mergeCell ref="C10:C14"/>
+    <mergeCell ref="A16:A58"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="C62:C72"/>
+    <mergeCell ref="D71:D72"/>
+    <mergeCell ref="D24:D29"/>
+    <mergeCell ref="D42:D45"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="C42:C47"/>
   </mergeCells>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
* * * 【2025/08/17 定例会】      実際は2025/8/31に実施
１．各自の立替分の精算
　　＊メイン口座の残額は、先月より48万円増えたが、偶数月に振込まれる下記保険金収入66万円によるものである。
　　 		国民厚生年金　		45
 			パナ年金　　　  	12
 			ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 	 9
　　　　従って、今月のメイン口座の支出は18万円前後ということになる？
　　＊共通口座の残額は、先月より30万円減ったが、新潟帰省（墓参，飯山出雲，川口やな、実家修理）の旅行イベントのためである。。
　　　　　(1)保険料
　　　　　(2)生活費
　　　　　　　　・小遣い振込			 	 7
　　　　　　　　・現金立替分				10			＊帰省中の現金立替分を含む
　　　　　　　　・その他カード引落分		 ?
　　　　　(3)イベント費
　　　　　　　　・新潟帰省　　　　　　　　　　　　　　　　　　　？

２．収支の確認
　　＊メイン口座は想定通り。
　　　 ただ楽天コード日4000円がここっから引き落とされていることが判明した。要修正。
　　＊共通口座の残額669万円で、ここまでの平均30万円程度で減少しているので、
　　　　このペースなら７か月後の年度末には459万円前後になる。
　　　　計画残高は399万円なのでイベント費は160万円しか残らない。
　　　　これから行う予定のリフォームの400万円，国内旅行（秋の金華山，畑毛）50?万円は厳しくなりそう。

３．メイン口座と共通口座のバランス確認
　　＊特になし

４．計画（ライフプラン.xlsx）の修正
　　＊特になし
</commit_message>
<xml_diff>
--- a/ライフプラン_猪飼.xlsx
+++ b/ライフプラン_猪飼.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC_USER\Documents\LocalLifeplanRepo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69ED5398-DEAC-40DB-A7A6-FDDD395D3F6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6505266-3ED1-4098-95CE-DB6112BD47D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{934FA03D-99BD-49E0-BFEC-291BD79F4879}"/>
   </bookViews>
@@ -679,7 +679,62 @@
         </r>
       </text>
     </comment>
+    <comment ref="G93" authorId="0" shapeId="0" xr:uid="{262036F5-01FA-4BC8-B8EB-1514CB55C6A6}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>PC_USER:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G94" authorId="0" shapeId="0" xr:uid="{69E2AA54-2427-4F59-AEE5-E8228FFFDD16}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>PC_USER:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="G107" authorId="0" shapeId="0" xr:uid="{38567A5A-08F1-44CE-8C1B-7B9A61C0360A}">
+      <text/>
+    </comment>
+    <comment ref="E108" authorId="0" shapeId="0" xr:uid="{0CFE7B6C-FEBF-4C82-A58B-E327835A20D7}">
       <text>
         <r>
           <rPr>
@@ -754,6 +809,70 @@
  全労済個人年金  + 2　
  ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 + 9
 nao</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G114" authorId="0" shapeId="0" xr:uid="{0F2950A9-8AE7-4919-82C2-D9C59D0C6A78}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>kaz
+ 東北電力配当金  + 1
+ 全労済東１      + 4
+ ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 + 9
+nao</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G115" authorId="0" shapeId="0" xr:uid="{AA4D0E19-713A-481C-B4AD-6D9DEF9AEC0C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>kaz
+ 国民厚生年金　　+45
+ パナ年金　　　  +12　
+ ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 + 9
+nao</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J115" authorId="0" shapeId="0" xr:uid="{C621A1A5-ABEA-449D-808A-68EDB182D85A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>PC_USER:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
         </r>
       </text>
     </comment>
@@ -857,6 +976,38 @@
           </rPr>
           <t>kazへ返済 -12 (ｶｲﾛ：6、CPAP：1、中山会：１。ﾋﾞｭｰ：1。医療費他)
 naoへ返済 -3（網代0.5、出雲＆瀬戸0.4、牛乳交通費食品等2）</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G134" authorId="0" shapeId="0" xr:uid="{536E0B11-8AD1-4BDA-A536-4C9DAB300E5A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>kazへ返済 -4 (新潟_網戸&amp;小嶋屋：1.1、医療費：1.4、ﾋﾞｭｰ：1。他)
+naoへ返済 -2.5（出雲；3，森永：0.3， 交通費返却：-0.7）</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G135" authorId="0" shapeId="0" xr:uid="{CAB7EF98-2301-4D34-AE07-4666B00D6496}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>kazへ返済 -7 (墓参：1、飯山出雲&amp;鮎：1.2、実家修理：1.6，ﾋﾞｭｰ：1。衣笠浜寿司：1.2、他：1)
+naoへ返済 -2.5（飯山出雲；2，森永：0.2， 町内祭:0.3）</t>
         </r>
       </text>
     </comment>
@@ -3745,109 +3896,6 @@
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" textRotation="255"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="42" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="1" applyBorder="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" textRotation="255"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" textRotation="255"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -3857,6 +3905,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" textRotation="255"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" textRotation="255"/>
@@ -3910,6 +3962,105 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" textRotation="255"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="42" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" textRotation="255"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="1" applyBorder="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5854,15 +6005,12 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>1076</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="4">
@@ -6101,7 +6249,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>1124</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -7341,6 +7489,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7348,7 +7497,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9306,7 +9454,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>691</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -9553,7 +9701,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>669</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -10796,6 +10944,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10803,7 +10952,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12757,7 +12905,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>1767</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -13004,7 +13152,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>1793</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -16446,12 +16594,12 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="128" t="s">
+      <c r="B1" s="99" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="129"/>
-      <c r="D1" s="129"/>
-      <c r="E1" s="130"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="101"/>
       <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
@@ -16552,13 +16700,13 @@
       <c r="AM1" s="4"/>
     </row>
     <row r="2" spans="1:39" ht="18.75" customHeight="1">
-      <c r="A2" s="99" t="s">
+      <c r="A2" s="102" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="133" t="s">
+      <c r="B2" s="105" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="140"/>
+      <c r="C2" s="112"/>
       <c r="D2" s="6" t="s">
         <v>5</v>
       </c>
@@ -16643,9 +16791,9 @@
       <c r="AM2" s="4"/>
     </row>
     <row r="3" spans="1:39" ht="19.5" thickBot="1">
-      <c r="A3" s="131"/>
-      <c r="B3" s="134"/>
-      <c r="C3" s="141"/>
+      <c r="A3" s="103"/>
+      <c r="B3" s="106"/>
+      <c r="C3" s="113"/>
       <c r="D3" s="9" t="s">
         <v>7</v>
       </c>
@@ -16746,11 +16894,11 @@
       <c r="AM3" s="4"/>
     </row>
     <row r="4" spans="1:39">
-      <c r="A4" s="131"/>
-      <c r="B4" s="133" t="s">
+      <c r="A4" s="103"/>
+      <c r="B4" s="105" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="142"/>
+      <c r="C4" s="114"/>
       <c r="D4" s="12" t="s">
         <v>10</v>
       </c>
@@ -16795,9 +16943,9 @@
       <c r="AM4" s="4"/>
     </row>
     <row r="5" spans="1:39">
-      <c r="A5" s="131"/>
-      <c r="B5" s="135"/>
-      <c r="C5" s="143"/>
+      <c r="A5" s="103"/>
+      <c r="B5" s="107"/>
+      <c r="C5" s="115"/>
       <c r="D5" s="15" t="s">
         <v>12</v>
       </c>
@@ -16842,9 +16990,9 @@
       <c r="AM5" s="4"/>
     </row>
     <row r="6" spans="1:39">
-      <c r="A6" s="131"/>
-      <c r="B6" s="135"/>
-      <c r="C6" s="143"/>
+      <c r="A6" s="103"/>
+      <c r="B6" s="107"/>
+      <c r="C6" s="115"/>
       <c r="D6" s="15"/>
       <c r="E6" s="16"/>
       <c r="F6" s="17"/>
@@ -16883,9 +17031,9 @@
       <c r="AM6" s="4"/>
     </row>
     <row r="7" spans="1:39">
-      <c r="A7" s="131"/>
-      <c r="B7" s="135"/>
-      <c r="C7" s="143"/>
+      <c r="A7" s="103"/>
+      <c r="B7" s="107"/>
+      <c r="C7" s="115"/>
       <c r="D7" s="15"/>
       <c r="E7" s="16"/>
       <c r="F7" s="17"/>
@@ -16924,9 +17072,9 @@
       <c r="AM7" s="4"/>
     </row>
     <row r="8" spans="1:39">
-      <c r="A8" s="131"/>
-      <c r="B8" s="136"/>
-      <c r="C8" s="144"/>
+      <c r="A8" s="103"/>
+      <c r="B8" s="108"/>
+      <c r="C8" s="116"/>
       <c r="D8" s="15"/>
       <c r="E8" s="16"/>
       <c r="F8" s="17"/>
@@ -16965,12 +17113,12 @@
       <c r="AM8" s="4"/>
     </row>
     <row r="9" spans="1:39" ht="19.5" thickBot="1">
-      <c r="A9" s="131"/>
-      <c r="B9" s="137" t="s">
+      <c r="A9" s="103"/>
+      <c r="B9" s="109" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="138"/>
-      <c r="D9" s="139"/>
+      <c r="C9" s="110"/>
+      <c r="D9" s="111"/>
       <c r="E9" s="18" t="s">
         <v>15</v>
       </c>
@@ -17106,11 +17254,11 @@
       <c r="AM9" s="4"/>
     </row>
     <row r="10" spans="1:39">
-      <c r="A10" s="131"/>
-      <c r="B10" s="133" t="s">
+      <c r="A10" s="103"/>
+      <c r="B10" s="105" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="142"/>
+      <c r="C10" s="114"/>
       <c r="D10" s="15" t="s">
         <v>17</v>
       </c>
@@ -17209,9 +17357,9 @@
       <c r="AM10" s="4"/>
     </row>
     <row r="11" spans="1:39">
-      <c r="A11" s="131"/>
-      <c r="B11" s="135"/>
-      <c r="C11" s="143"/>
+      <c r="A11" s="103"/>
+      <c r="B11" s="107"/>
+      <c r="C11" s="115"/>
       <c r="D11" s="15" t="s">
         <v>19</v>
       </c>
@@ -17261,9 +17409,9 @@
       <c r="AM11" s="4"/>
     </row>
     <row r="12" spans="1:39">
-      <c r="A12" s="131"/>
-      <c r="B12" s="135"/>
-      <c r="C12" s="143"/>
+      <c r="A12" s="103"/>
+      <c r="B12" s="107"/>
+      <c r="C12" s="115"/>
       <c r="D12" s="15" t="s">
         <v>21</v>
       </c>
@@ -17335,9 +17483,9 @@
       <c r="AM12" s="4"/>
     </row>
     <row r="13" spans="1:39">
-      <c r="A13" s="131"/>
-      <c r="B13" s="135"/>
-      <c r="C13" s="143"/>
+      <c r="A13" s="103"/>
+      <c r="B13" s="107"/>
+      <c r="C13" s="115"/>
       <c r="D13" s="15" t="s">
         <v>22</v>
       </c>
@@ -17386,9 +17534,9 @@
       <c r="AM13" s="4"/>
     </row>
     <row r="14" spans="1:39">
-      <c r="A14" s="131"/>
-      <c r="B14" s="136"/>
-      <c r="C14" s="144"/>
+      <c r="A14" s="103"/>
+      <c r="B14" s="108"/>
+      <c r="C14" s="116"/>
       <c r="D14" s="15"/>
       <c r="E14" s="16"/>
       <c r="F14" s="23"/>
@@ -17427,12 +17575,12 @@
       <c r="AM14" s="4"/>
     </row>
     <row r="15" spans="1:39" ht="19.5" thickBot="1">
-      <c r="A15" s="132"/>
-      <c r="B15" s="137" t="s">
+      <c r="A15" s="104"/>
+      <c r="B15" s="109" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="138"/>
-      <c r="D15" s="139"/>
+      <c r="C15" s="110"/>
+      <c r="D15" s="111"/>
       <c r="E15" s="18" t="s">
         <v>25</v>
       </c>
@@ -17568,16 +17716,16 @@
       <c r="AM15" s="4"/>
     </row>
     <row r="16" spans="1:39">
-      <c r="A16" s="99" t="s">
+      <c r="A16" s="102" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="126" t="s">
+      <c r="B16" s="136" t="s">
         <v>132</v>
       </c>
       <c r="C16" s="118" t="s">
         <v>108</v>
       </c>
-      <c r="D16" s="119" t="s">
+      <c r="D16" s="120" t="s">
         <v>112</v>
       </c>
       <c r="E16" s="16" t="s">
@@ -17659,10 +17807,10 @@
       <c r="AM16" s="4"/>
     </row>
     <row r="17" spans="1:39">
-      <c r="A17" s="100"/>
-      <c r="B17" s="124"/>
-      <c r="C17" s="107"/>
-      <c r="D17" s="107"/>
+      <c r="A17" s="138"/>
+      <c r="B17" s="134"/>
+      <c r="C17" s="119"/>
+      <c r="D17" s="119"/>
       <c r="E17" s="16" t="s">
         <v>30</v>
       </c>
@@ -17748,12 +17896,12 @@
       <c r="AM17" s="4"/>
     </row>
     <row r="18" spans="1:39">
-      <c r="A18" s="100"/>
-      <c r="B18" s="124"/>
-      <c r="C18" s="110" t="s">
+      <c r="A18" s="138"/>
+      <c r="B18" s="134"/>
+      <c r="C18" s="121" t="s">
         <v>109</v>
       </c>
-      <c r="D18" s="111" t="s">
+      <c r="D18" s="123" t="s">
         <v>114</v>
       </c>
       <c r="E18" s="13" t="s">
@@ -17835,10 +17983,10 @@
       <c r="AM18" s="27"/>
     </row>
     <row r="19" spans="1:39">
-      <c r="A19" s="100"/>
-      <c r="B19" s="124"/>
-      <c r="C19" s="112"/>
-      <c r="D19" s="112"/>
+      <c r="A19" s="138"/>
+      <c r="B19" s="134"/>
+      <c r="C19" s="122"/>
+      <c r="D19" s="122"/>
       <c r="E19" s="16" t="s">
         <v>28</v>
       </c>
@@ -17906,10 +18054,10 @@
       <c r="AM19" s="27"/>
     </row>
     <row r="20" spans="1:39">
-      <c r="A20" s="100"/>
-      <c r="B20" s="124"/>
-      <c r="C20" s="112"/>
-      <c r="D20" s="107"/>
+      <c r="A20" s="138"/>
+      <c r="B20" s="134"/>
+      <c r="C20" s="122"/>
+      <c r="D20" s="119"/>
       <c r="E20" s="16" t="s">
         <v>29</v>
       </c>
@@ -17959,9 +18107,9 @@
       <c r="AM20" s="27"/>
     </row>
     <row r="21" spans="1:39">
-      <c r="A21" s="100"/>
-      <c r="B21" s="124"/>
-      <c r="C21" s="107"/>
+      <c r="A21" s="138"/>
+      <c r="B21" s="134"/>
+      <c r="C21" s="119"/>
       <c r="D21" s="57" t="s">
         <v>115</v>
       </c>
@@ -18012,9 +18160,9 @@
       <c r="AM21" s="27"/>
     </row>
     <row r="22" spans="1:39">
-      <c r="A22" s="100"/>
-      <c r="B22" s="124"/>
-      <c r="C22" s="110" t="s">
+      <c r="A22" s="138"/>
+      <c r="B22" s="134"/>
+      <c r="C22" s="121" t="s">
         <v>110</v>
       </c>
       <c r="D22" s="57" t="s">
@@ -18059,9 +18207,9 @@
       <c r="AM22" s="27"/>
     </row>
     <row r="23" spans="1:39">
-      <c r="A23" s="100"/>
-      <c r="B23" s="124"/>
-      <c r="C23" s="107"/>
+      <c r="A23" s="138"/>
+      <c r="B23" s="134"/>
+      <c r="C23" s="119"/>
       <c r="D23" s="57" t="s">
         <v>117</v>
       </c>
@@ -18104,12 +18252,12 @@
       <c r="AM23" s="27"/>
     </row>
     <row r="24" spans="1:39">
-      <c r="A24" s="100"/>
-      <c r="B24" s="124"/>
-      <c r="C24" s="110" t="s">
+      <c r="A24" s="138"/>
+      <c r="B24" s="134"/>
+      <c r="C24" s="121" t="s">
         <v>111</v>
       </c>
-      <c r="D24" s="111" t="s">
+      <c r="D24" s="123" t="s">
         <v>118</v>
       </c>
       <c r="E24" s="16" t="s">
@@ -18191,10 +18339,10 @@
       <c r="AM24" s="27"/>
     </row>
     <row r="25" spans="1:39">
-      <c r="A25" s="100"/>
-      <c r="B25" s="124"/>
-      <c r="C25" s="112"/>
-      <c r="D25" s="112"/>
+      <c r="A25" s="138"/>
+      <c r="B25" s="134"/>
+      <c r="C25" s="122"/>
+      <c r="D25" s="122"/>
       <c r="E25" s="16" t="s">
         <v>33</v>
       </c>
@@ -18286,10 +18434,10 @@
       <c r="AM25" s="27"/>
     </row>
     <row r="26" spans="1:39">
-      <c r="A26" s="100"/>
-      <c r="B26" s="124"/>
-      <c r="C26" s="112"/>
-      <c r="D26" s="112"/>
+      <c r="A26" s="138"/>
+      <c r="B26" s="134"/>
+      <c r="C26" s="122"/>
+      <c r="D26" s="122"/>
       <c r="E26" s="16" t="s">
         <v>34</v>
       </c>
@@ -18331,10 +18479,10 @@
       <c r="AM26" s="27"/>
     </row>
     <row r="27" spans="1:39">
-      <c r="A27" s="100"/>
-      <c r="B27" s="124"/>
-      <c r="C27" s="112"/>
-      <c r="D27" s="112"/>
+      <c r="A27" s="138"/>
+      <c r="B27" s="134"/>
+      <c r="C27" s="122"/>
+      <c r="D27" s="122"/>
       <c r="E27" s="29" t="s">
         <v>35</v>
       </c>
@@ -18376,10 +18524,10 @@
       <c r="AM27" s="27"/>
     </row>
     <row r="28" spans="1:39">
-      <c r="A28" s="100"/>
-      <c r="B28" s="124"/>
-      <c r="C28" s="112"/>
-      <c r="D28" s="112"/>
+      <c r="A28" s="138"/>
+      <c r="B28" s="134"/>
+      <c r="C28" s="122"/>
+      <c r="D28" s="122"/>
       <c r="E28" s="16" t="s">
         <v>36</v>
       </c>
@@ -18439,10 +18587,10 @@
       <c r="AM28" s="27"/>
     </row>
     <row r="29" spans="1:39">
-      <c r="A29" s="100"/>
-      <c r="B29" s="124"/>
-      <c r="C29" s="112"/>
-      <c r="D29" s="107"/>
+      <c r="A29" s="138"/>
+      <c r="B29" s="134"/>
+      <c r="C29" s="122"/>
+      <c r="D29" s="119"/>
       <c r="E29" s="86" t="s">
         <v>120</v>
       </c>
@@ -18484,9 +18632,9 @@
       <c r="AM29" s="27"/>
     </row>
     <row r="30" spans="1:39">
-      <c r="A30" s="100"/>
-      <c r="B30" s="124"/>
-      <c r="C30" s="112"/>
+      <c r="A30" s="138"/>
+      <c r="B30" s="134"/>
+      <c r="C30" s="122"/>
       <c r="D30" s="57" t="s">
         <v>122</v>
       </c>
@@ -18529,9 +18677,9 @@
       <c r="AM30" s="27"/>
     </row>
     <row r="31" spans="1:39">
-      <c r="A31" s="100"/>
-      <c r="B31" s="125"/>
-      <c r="C31" s="107"/>
+      <c r="A31" s="138"/>
+      <c r="B31" s="135"/>
+      <c r="C31" s="119"/>
       <c r="D31" s="57" t="s">
         <v>123</v>
       </c>
@@ -18574,11 +18722,11 @@
       <c r="AM31" s="27"/>
     </row>
     <row r="32" spans="1:39">
-      <c r="A32" s="100"/>
-      <c r="B32" s="115" t="s">
+      <c r="A32" s="138"/>
+      <c r="B32" s="143" t="s">
         <v>131</v>
       </c>
-      <c r="C32" s="108"/>
+      <c r="C32" s="124"/>
       <c r="D32" s="17" t="s">
         <v>128</v>
       </c>
@@ -18677,9 +18825,9 @@
       <c r="AM32" s="27"/>
     </row>
     <row r="33" spans="1:39">
-      <c r="A33" s="100"/>
-      <c r="B33" s="116"/>
-      <c r="C33" s="105"/>
+      <c r="A33" s="138"/>
+      <c r="B33" s="144"/>
+      <c r="C33" s="126"/>
       <c r="D33" s="17" t="s">
         <v>129</v>
       </c>
@@ -18754,12 +18902,12 @@
       <c r="AM33" s="27"/>
     </row>
     <row r="34" spans="1:39">
-      <c r="A34" s="100"/>
-      <c r="B34" s="102" t="s">
+      <c r="A34" s="138"/>
+      <c r="B34" s="127" t="s">
         <v>9</v>
       </c>
-      <c r="C34" s="104"/>
-      <c r="D34" s="106"/>
+      <c r="C34" s="130"/>
+      <c r="D34" s="140"/>
       <c r="E34" s="34" t="str">
         <f t="shared" ref="E34:AK34" si="2">E4</f>
         <v>新潟実家の売却益　（妙子と折半）</v>
@@ -18896,10 +19044,10 @@
       <c r="AM34" s="27"/>
     </row>
     <row r="35" spans="1:39">
-      <c r="A35" s="100"/>
-      <c r="B35" s="103"/>
-      <c r="C35" s="105"/>
-      <c r="D35" s="107"/>
+      <c r="A35" s="138"/>
+      <c r="B35" s="129"/>
+      <c r="C35" s="126"/>
+      <c r="D35" s="119"/>
       <c r="E35" s="34" t="str">
         <f t="shared" ref="E35:AK35" si="3">E5</f>
         <v>横浜マンションの売却益</v>
@@ -19036,7 +19184,7 @@
       <c r="AM35" s="27"/>
     </row>
     <row r="36" spans="1:39" ht="19.5" thickBot="1">
-      <c r="A36" s="100"/>
+      <c r="A36" s="138"/>
       <c r="B36" s="35" t="s">
         <v>38</v>
       </c>
@@ -19175,8 +19323,8 @@
       <c r="AM36" s="27"/>
     </row>
     <row r="37" spans="1:39">
-      <c r="A37" s="100"/>
-      <c r="B37" s="123" t="s">
+      <c r="A37" s="138"/>
+      <c r="B37" s="133" t="s">
         <v>133</v>
       </c>
       <c r="C37" s="8" t="s">
@@ -19226,9 +19374,9 @@
       <c r="AM37" s="4"/>
     </row>
     <row r="38" spans="1:39">
-      <c r="A38" s="100"/>
-      <c r="B38" s="124"/>
-      <c r="C38" s="110" t="s">
+      <c r="A38" s="138"/>
+      <c r="B38" s="134"/>
+      <c r="C38" s="121" t="s">
         <v>109</v>
       </c>
       <c r="D38" s="57" t="s">
@@ -19273,9 +19421,9 @@
       <c r="AM38" s="4"/>
     </row>
     <row r="39" spans="1:39">
-      <c r="A39" s="100"/>
-      <c r="B39" s="124"/>
-      <c r="C39" s="107"/>
+      <c r="A39" s="138"/>
+      <c r="B39" s="134"/>
+      <c r="C39" s="119"/>
       <c r="D39" s="57" t="s">
         <v>115</v>
       </c>
@@ -19318,9 +19466,9 @@
       <c r="AM39" s="4"/>
     </row>
     <row r="40" spans="1:39">
-      <c r="A40" s="100"/>
-      <c r="B40" s="124"/>
-      <c r="C40" s="110" t="s">
+      <c r="A40" s="138"/>
+      <c r="B40" s="134"/>
+      <c r="C40" s="121" t="s">
         <v>110</v>
       </c>
       <c r="D40" s="57" t="s">
@@ -19421,9 +19569,9 @@
       <c r="AM40" s="27"/>
     </row>
     <row r="41" spans="1:39">
-      <c r="A41" s="100"/>
-      <c r="B41" s="124"/>
-      <c r="C41" s="107"/>
+      <c r="A41" s="138"/>
+      <c r="B41" s="134"/>
+      <c r="C41" s="119"/>
       <c r="D41" s="57" t="s">
         <v>117</v>
       </c>
@@ -19466,12 +19614,12 @@
       <c r="AM41" s="4"/>
     </row>
     <row r="42" spans="1:39">
-      <c r="A42" s="100"/>
-      <c r="B42" s="124"/>
-      <c r="C42" s="110" t="s">
+      <c r="A42" s="138"/>
+      <c r="B42" s="134"/>
+      <c r="C42" s="121" t="s">
         <v>111</v>
       </c>
-      <c r="D42" s="111" t="s">
+      <c r="D42" s="123" t="s">
         <v>118</v>
       </c>
       <c r="E42" s="16" t="s">
@@ -19517,10 +19665,10 @@
       <c r="AM42" s="27"/>
     </row>
     <row r="43" spans="1:39">
-      <c r="A43" s="100"/>
-      <c r="B43" s="124"/>
-      <c r="C43" s="112"/>
-      <c r="D43" s="112"/>
+      <c r="A43" s="138"/>
+      <c r="B43" s="134"/>
+      <c r="C43" s="122"/>
+      <c r="D43" s="122"/>
       <c r="E43" s="16" t="s">
         <v>49</v>
       </c>
@@ -19600,10 +19748,10 @@
       <c r="AM43" s="27"/>
     </row>
     <row r="44" spans="1:39">
-      <c r="A44" s="100"/>
-      <c r="B44" s="124"/>
-      <c r="C44" s="112"/>
-      <c r="D44" s="112"/>
+      <c r="A44" s="138"/>
+      <c r="B44" s="134"/>
+      <c r="C44" s="122"/>
+      <c r="D44" s="122"/>
       <c r="E44" s="16" t="s">
         <v>50</v>
       </c>
@@ -19675,10 +19823,10 @@
       <c r="AM44" s="27"/>
     </row>
     <row r="45" spans="1:39">
-      <c r="A45" s="100"/>
-      <c r="B45" s="124"/>
-      <c r="C45" s="112"/>
-      <c r="D45" s="107"/>
+      <c r="A45" s="138"/>
+      <c r="B45" s="134"/>
+      <c r="C45" s="122"/>
+      <c r="D45" s="119"/>
       <c r="E45" s="86" t="s">
         <v>124</v>
       </c>
@@ -19728,9 +19876,9 @@
       <c r="AM45" s="27"/>
     </row>
     <row r="46" spans="1:39">
-      <c r="A46" s="100"/>
-      <c r="B46" s="124"/>
-      <c r="C46" s="112"/>
+      <c r="A46" s="138"/>
+      <c r="B46" s="134"/>
+      <c r="C46" s="122"/>
       <c r="D46" s="57" t="s">
         <v>122</v>
       </c>
@@ -19823,9 +19971,9 @@
       <c r="AM46" s="27"/>
     </row>
     <row r="47" spans="1:39">
-      <c r="A47" s="100"/>
-      <c r="B47" s="125"/>
-      <c r="C47" s="107"/>
+      <c r="A47" s="138"/>
+      <c r="B47" s="135"/>
+      <c r="C47" s="119"/>
       <c r="D47" s="57" t="s">
         <v>123</v>
       </c>
@@ -19868,7 +20016,7 @@
       <c r="AM47" s="4"/>
     </row>
     <row r="48" spans="1:39">
-      <c r="A48" s="100"/>
+      <c r="A48" s="138"/>
       <c r="B48" s="66" t="s">
         <v>45</v>
       </c>
@@ -19953,7 +20101,7 @@
       <c r="AM48" s="27"/>
     </row>
     <row r="49" spans="1:39">
-      <c r="A49" s="100"/>
+      <c r="A49" s="138"/>
       <c r="B49" s="66" t="s">
         <v>52</v>
       </c>
@@ -20054,7 +20202,7 @@
       <c r="AM49" s="27"/>
     </row>
     <row r="50" spans="1:39">
-      <c r="A50" s="100"/>
+      <c r="A50" s="138"/>
       <c r="B50" s="66" t="s">
         <v>54</v>
       </c>
@@ -20155,11 +20303,11 @@
       <c r="AM50" s="27"/>
     </row>
     <row r="51" spans="1:39">
-      <c r="A51" s="100"/>
-      <c r="B51" s="122" t="s">
+      <c r="A51" s="138"/>
+      <c r="B51" s="132" t="s">
         <v>125</v>
       </c>
-      <c r="C51" s="108"/>
+      <c r="C51" s="124"/>
       <c r="D51" s="15" t="s">
         <v>43</v>
       </c>
@@ -20242,9 +20390,9 @@
       <c r="AM51" s="27"/>
     </row>
     <row r="52" spans="1:39">
-      <c r="A52" s="100"/>
-      <c r="B52" s="120"/>
-      <c r="C52" s="109"/>
+      <c r="A52" s="138"/>
+      <c r="B52" s="128"/>
+      <c r="C52" s="125"/>
       <c r="D52" s="15" t="s">
         <v>39</v>
       </c>
@@ -20289,9 +20437,9 @@
       <c r="AM52" s="27"/>
     </row>
     <row r="53" spans="1:39">
-      <c r="A53" s="100"/>
-      <c r="B53" s="103"/>
-      <c r="C53" s="105"/>
+      <c r="A53" s="138"/>
+      <c r="B53" s="129"/>
+      <c r="C53" s="126"/>
       <c r="D53" s="15" t="s">
         <v>41</v>
       </c>
@@ -20390,7 +20538,7 @@
       <c r="AM53" s="27"/>
     </row>
     <row r="54" spans="1:39">
-      <c r="A54" s="100"/>
+      <c r="A54" s="138"/>
       <c r="B54" s="84" t="s">
         <v>141</v>
       </c>
@@ -20493,11 +20641,11 @@
       <c r="AM54" s="27"/>
     </row>
     <row r="55" spans="1:39">
-      <c r="A55" s="100"/>
-      <c r="B55" s="113" t="s">
+      <c r="A55" s="138"/>
+      <c r="B55" s="141" t="s">
         <v>148</v>
       </c>
-      <c r="C55" s="114"/>
+      <c r="C55" s="142"/>
       <c r="D55" s="78" t="s">
         <v>127</v>
       </c>
@@ -20620,7 +20768,7 @@
       <c r="AM55" s="27"/>
     </row>
     <row r="56" spans="1:39">
-      <c r="A56" s="100"/>
+      <c r="A56" s="138"/>
       <c r="B56" s="67" t="s">
         <v>58</v>
       </c>
@@ -20749,7 +20897,7 @@
       <c r="AM56" s="27"/>
     </row>
     <row r="57" spans="1:39">
-      <c r="A57" s="100"/>
+      <c r="A57" s="138"/>
       <c r="B57" s="67" t="s">
         <v>60</v>
       </c>
@@ -20876,7 +21024,7 @@
       <c r="AM57" s="27"/>
     </row>
     <row r="58" spans="1:39" ht="19.5" thickBot="1">
-      <c r="A58" s="101"/>
+      <c r="A58" s="139"/>
       <c r="B58" s="61" t="s">
         <v>61</v>
       </c>
@@ -21005,7 +21153,7 @@
       <c r="AM58" s="27"/>
     </row>
     <row r="59" spans="1:39" ht="18.75" customHeight="1">
-      <c r="A59" s="99" t="s">
+      <c r="A59" s="102" t="s">
         <v>62</v>
       </c>
       <c r="B59" s="81" t="s">
@@ -21139,7 +21287,7 @@
       <c r="AM59" s="27"/>
     </row>
     <row r="60" spans="1:39" ht="19.5" thickBot="1">
-      <c r="A60" s="127"/>
+      <c r="A60" s="137"/>
       <c r="B60" s="61" t="s">
         <v>38</v>
       </c>
@@ -21269,7 +21417,7 @@
       <c r="AM60" s="27"/>
     </row>
     <row r="61" spans="1:39">
-      <c r="A61" s="127"/>
+      <c r="A61" s="137"/>
       <c r="B61" s="68" t="s">
         <v>138</v>
       </c>
@@ -21320,11 +21468,11 @@
       <c r="AM61" s="27"/>
     </row>
     <row r="62" spans="1:39">
-      <c r="A62" s="127"/>
-      <c r="B62" s="121" t="s">
+      <c r="A62" s="137"/>
+      <c r="B62" s="131" t="s">
         <v>125</v>
       </c>
-      <c r="C62" s="108"/>
+      <c r="C62" s="124"/>
       <c r="D62" s="72" t="s">
         <v>64</v>
       </c>
@@ -21423,9 +21571,9 @@
       <c r="AM62" s="27"/>
     </row>
     <row r="63" spans="1:39">
-      <c r="A63" s="127"/>
-      <c r="B63" s="120"/>
-      <c r="C63" s="109"/>
+      <c r="A63" s="137"/>
+      <c r="B63" s="128"/>
+      <c r="C63" s="125"/>
       <c r="D63" s="15" t="s">
         <v>66</v>
       </c>
@@ -21524,9 +21672,9 @@
       <c r="AM63" s="27"/>
     </row>
     <row r="64" spans="1:39">
-      <c r="A64" s="127"/>
-      <c r="B64" s="120"/>
-      <c r="C64" s="109"/>
+      <c r="A64" s="137"/>
+      <c r="B64" s="128"/>
+      <c r="C64" s="125"/>
       <c r="D64" s="15" t="s">
         <v>68</v>
       </c>
@@ -21625,9 +21773,9 @@
       <c r="AM64" s="27"/>
     </row>
     <row r="65" spans="1:39">
-      <c r="A65" s="127"/>
-      <c r="B65" s="120"/>
-      <c r="C65" s="109"/>
+      <c r="A65" s="137"/>
+      <c r="B65" s="128"/>
+      <c r="C65" s="125"/>
       <c r="D65" s="15" t="s">
         <v>70</v>
       </c>
@@ -21726,9 +21874,9 @@
       <c r="AM65" s="27"/>
     </row>
     <row r="66" spans="1:39">
-      <c r="A66" s="127"/>
-      <c r="B66" s="120"/>
-      <c r="C66" s="109"/>
+      <c r="A66" s="137"/>
+      <c r="B66" s="128"/>
+      <c r="C66" s="125"/>
       <c r="D66" s="15" t="s">
         <v>54</v>
       </c>
@@ -21827,9 +21975,9 @@
       <c r="AM66" s="27"/>
     </row>
     <row r="67" spans="1:39">
-      <c r="A67" s="127"/>
-      <c r="B67" s="120"/>
-      <c r="C67" s="109"/>
+      <c r="A67" s="137"/>
+      <c r="B67" s="128"/>
+      <c r="C67" s="125"/>
       <c r="D67" s="15" t="s">
         <v>73</v>
       </c>
@@ -21928,9 +22076,9 @@
       <c r="AM67" s="27"/>
     </row>
     <row r="68" spans="1:39">
-      <c r="A68" s="127"/>
-      <c r="B68" s="120"/>
-      <c r="C68" s="109"/>
+      <c r="A68" s="137"/>
+      <c r="B68" s="128"/>
+      <c r="C68" s="125"/>
       <c r="D68" s="15" t="s">
         <v>75</v>
       </c>
@@ -22029,9 +22177,9 @@
       <c r="AM68" s="27"/>
     </row>
     <row r="69" spans="1:39">
-      <c r="A69" s="127"/>
-      <c r="B69" s="120"/>
-      <c r="C69" s="109"/>
+      <c r="A69" s="137"/>
+      <c r="B69" s="128"/>
+      <c r="C69" s="125"/>
       <c r="D69" s="15" t="s">
         <v>77</v>
       </c>
@@ -22130,9 +22278,9 @@
       <c r="AM69" s="27"/>
     </row>
     <row r="70" spans="1:39">
-      <c r="A70" s="127"/>
-      <c r="B70" s="120"/>
-      <c r="C70" s="109"/>
+      <c r="A70" s="137"/>
+      <c r="B70" s="128"/>
+      <c r="C70" s="125"/>
       <c r="D70" s="15" t="s">
         <v>79</v>
       </c>
@@ -22231,10 +22379,10 @@
       <c r="AM70" s="27"/>
     </row>
     <row r="71" spans="1:39">
-      <c r="A71" s="127"/>
-      <c r="B71" s="120"/>
-      <c r="C71" s="109"/>
-      <c r="D71" s="110" t="s">
+      <c r="A71" s="137"/>
+      <c r="B71" s="128"/>
+      <c r="C71" s="125"/>
+      <c r="D71" s="121" t="s">
         <v>82</v>
       </c>
       <c r="E71" s="16" t="s">
@@ -22336,10 +22484,10 @@
       <c r="AM71" s="27"/>
     </row>
     <row r="72" spans="1:39">
-      <c r="A72" s="127"/>
-      <c r="B72" s="103"/>
-      <c r="C72" s="105"/>
-      <c r="D72" s="107"/>
+      <c r="A72" s="137"/>
+      <c r="B72" s="129"/>
+      <c r="C72" s="126"/>
+      <c r="D72" s="119"/>
       <c r="E72" s="16" t="s">
         <v>84</v>
       </c>
@@ -22439,11 +22587,11 @@
       <c r="AM72" s="27"/>
     </row>
     <row r="73" spans="1:39">
-      <c r="A73" s="127"/>
-      <c r="B73" s="102" t="s">
+      <c r="A73" s="137"/>
+      <c r="B73" s="127" t="s">
         <v>16</v>
       </c>
-      <c r="C73" s="104"/>
+      <c r="C73" s="130"/>
       <c r="D73" s="33" t="s">
         <v>134</v>
       </c>
@@ -22573,9 +22721,9 @@
       <c r="AM73" s="27"/>
     </row>
     <row r="74" spans="1:39">
-      <c r="A74" s="127"/>
-      <c r="B74" s="120"/>
-      <c r="C74" s="109"/>
+      <c r="A74" s="137"/>
+      <c r="B74" s="128"/>
+      <c r="C74" s="125"/>
       <c r="D74" s="33" t="s">
         <v>135</v>
       </c>
@@ -22705,9 +22853,9 @@
       <c r="AM74" s="27"/>
     </row>
     <row r="75" spans="1:39">
-      <c r="A75" s="127"/>
-      <c r="B75" s="120"/>
-      <c r="C75" s="109"/>
+      <c r="A75" s="137"/>
+      <c r="B75" s="128"/>
+      <c r="C75" s="125"/>
       <c r="D75" s="33" t="s">
         <v>136</v>
       </c>
@@ -22837,9 +22985,9 @@
       <c r="AM75" s="27"/>
     </row>
     <row r="76" spans="1:39">
-      <c r="A76" s="127"/>
-      <c r="B76" s="103"/>
-      <c r="C76" s="105"/>
+      <c r="A76" s="137"/>
+      <c r="B76" s="129"/>
+      <c r="C76" s="126"/>
       <c r="D76" s="33" t="s">
         <v>137</v>
       </c>
@@ -22969,7 +23117,7 @@
       <c r="AM76" s="27"/>
     </row>
     <row r="77" spans="1:39">
-      <c r="A77" s="127"/>
+      <c r="A77" s="137"/>
       <c r="B77" s="67" t="s">
         <v>58</v>
       </c>
@@ -23099,7 +23247,7 @@
       <c r="AM77" s="27"/>
     </row>
     <row r="78" spans="1:39">
-      <c r="A78" s="127"/>
+      <c r="A78" s="137"/>
       <c r="B78" s="67" t="s">
         <v>60</v>
       </c>
@@ -23358,7 +23506,7 @@
       <c r="AM79" s="27"/>
     </row>
     <row r="80" spans="1:39">
-      <c r="A80" s="99" t="s">
+      <c r="A80" s="102" t="s">
         <v>89</v>
       </c>
       <c r="B80" s="59" t="s">
@@ -24186,9 +24334,9 @@
       <c r="F94" s="55" t="s">
         <v>99</v>
       </c>
-      <c r="G94" s="56" t="e">
+      <c r="G94" s="56">
         <f t="shared" ref="G94:AK94" si="23">G114+G134</f>
-        <v>#N/A</v>
+        <v>1767</v>
       </c>
       <c r="H94" s="57" t="e">
         <f t="shared" si="23"/>
@@ -24315,9 +24463,9 @@
       <c r="F95" s="55" t="s">
         <v>100</v>
       </c>
-      <c r="G95" s="56" t="e">
+      <c r="G95" s="56">
         <f t="shared" ref="G95:AK95" si="24">G115+G135</f>
-        <v>#N/A</v>
+        <v>1793</v>
       </c>
       <c r="H95" s="57" t="e">
         <f t="shared" si="24"/>
@@ -24569,7 +24717,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="97" spans="6:37">
+    <row r="97" spans="5:37">
       <c r="F97" s="55" t="s">
         <v>102</v>
       </c>
@@ -24698,7 +24846,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="98" spans="6:37">
+    <row r="98" spans="5:37">
       <c r="F98" s="55" t="s">
         <v>103</v>
       </c>
@@ -24827,7 +24975,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="99" spans="6:37">
+    <row r="99" spans="5:37">
       <c r="F99" s="89" t="s">
         <v>104</v>
       </c>
@@ -24956,7 +25104,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="100" spans="6:37">
+    <row r="100" spans="5:37">
       <c r="F100" s="89" t="s">
         <v>93</v>
       </c>
@@ -25085,7 +25233,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="101" spans="6:37">
+    <row r="101" spans="5:37">
       <c r="F101" s="55" t="s">
         <v>94</v>
       </c>
@@ -25214,7 +25362,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="102" spans="6:37" ht="19.5" thickBot="1">
+    <row r="102" spans="5:37" ht="19.5" thickBot="1">
       <c r="F102" s="95" t="s">
         <v>95</v>
       </c>
@@ -25343,7 +25491,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="103" spans="6:37">
+    <row r="103" spans="5:37">
       <c r="F103" s="67" t="s">
         <v>105</v>
       </c>
@@ -25472,19 +25620,46 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="6:37" ht="19.5" thickBot="1">
+    <row r="104" spans="5:37" ht="19.5" thickBot="1">
       <c r="F104" s="61" t="s">
         <v>106</v>
       </c>
-      <c r="G104" s="45"/>
-      <c r="H104" s="41"/>
-      <c r="I104" s="41"/>
-      <c r="J104" s="41"/>
-      <c r="K104" s="41"/>
-      <c r="L104" s="41"/>
-      <c r="M104" s="41"/>
-      <c r="N104" s="41"/>
-      <c r="O104" s="41"/>
+      <c r="G104" s="45" t="e">
+        <f>G103-G99</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H104" s="41" t="e">
+        <f t="shared" ref="H104:O104" si="33">H103-H99</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I104" s="41" t="e">
+        <f t="shared" si="33"/>
+        <v>#N/A</v>
+      </c>
+      <c r="J104" s="41" t="e">
+        <f t="shared" si="33"/>
+        <v>#N/A</v>
+      </c>
+      <c r="K104" s="41" t="e">
+        <f t="shared" si="33"/>
+        <v>#N/A</v>
+      </c>
+      <c r="L104" s="41" t="e">
+        <f t="shared" si="33"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M104" s="41" t="e">
+        <f t="shared" si="33"/>
+        <v>#N/A</v>
+      </c>
+      <c r="N104" s="41" t="e">
+        <f t="shared" si="33"/>
+        <v>#N/A</v>
+      </c>
+      <c r="O104" s="41" t="e">
+        <f t="shared" si="33"/>
+        <v>#N/A</v>
+      </c>
       <c r="P104" s="41"/>
       <c r="Q104" s="41"/>
       <c r="R104" s="41"/>
@@ -25508,14 +25683,14 @@
       <c r="AJ104" s="41"/>
       <c r="AK104" s="42"/>
     </row>
-    <row r="107" spans="6:37"/>
-    <row r="108" spans="6:37" ht="24">
+    <row r="107" spans="5:37"/>
+    <row r="108" spans="5:37" ht="24">
       <c r="F108" s="54" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="109" spans="6:37" ht="19.5" thickBot="1"/>
-    <row r="110" spans="6:37" ht="19.5" thickBot="1">
+    <row r="109" spans="5:37" ht="19.5" thickBot="1"/>
+    <row r="110" spans="5:37" ht="19.5" thickBot="1">
       <c r="F110" s="92" t="s">
         <v>107</v>
       </c>
@@ -25613,7 +25788,7 @@
         <v>2055</v>
       </c>
     </row>
-    <row r="111" spans="6:37">
+    <row r="111" spans="5:37">
       <c r="F111" s="88" t="s">
         <v>96</v>
       </c>
@@ -25712,7 +25887,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="112" spans="6:37">
+    <row r="112" spans="5:37">
       <c r="F112" s="55" t="s">
         <v>97</v>
       </c>
@@ -25912,8 +26087,8 @@
       <c r="F114" s="55" t="s">
         <v>99</v>
       </c>
-      <c r="G114" s="56" t="e">
-        <v>#N/A</v>
+      <c r="G114" s="56">
+        <v>1076</v>
       </c>
       <c r="H114" s="57" t="e">
         <v>#N/A</v>
@@ -25921,9 +26096,7 @@
       <c r="I114" s="57" t="e">
         <v>#N/A</v>
       </c>
-      <c r="J114" s="57" t="e">
-        <v>#N/A</v>
-      </c>
+      <c r="J114" s="57"/>
       <c r="K114" s="57" t="e">
         <v>#N/A</v>
       </c>
@@ -26010,8 +26183,8 @@
       <c r="F115" s="55" t="s">
         <v>100</v>
       </c>
-      <c r="G115" s="56" t="e">
-        <v>#N/A</v>
+      <c r="G115" s="56">
+        <v>1124</v>
       </c>
       <c r="H115" s="57" t="e">
         <v>#N/A</v>
@@ -26795,127 +26968,127 @@
         <v>105</v>
       </c>
       <c r="G123" s="46">
-        <f t="shared" ref="G123:AK123" si="33">G58</f>
+        <f t="shared" ref="G123:AK123" si="34">G58</f>
         <v>651</v>
       </c>
       <c r="H123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>551</v>
       </c>
       <c r="I123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>349</v>
       </c>
       <c r="J123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>257</v>
       </c>
       <c r="K123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>237</v>
       </c>
       <c r="L123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>105</v>
       </c>
       <c r="M123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>103</v>
       </c>
       <c r="N123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>81</v>
       </c>
       <c r="O123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>59</v>
       </c>
       <c r="P123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>107</v>
       </c>
       <c r="Q123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>-195</v>
       </c>
       <c r="R123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>-197</v>
       </c>
       <c r="S123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>-279</v>
       </c>
       <c r="T123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>-341</v>
       </c>
       <c r="U123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>-502</v>
       </c>
       <c r="V123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>-653</v>
       </c>
       <c r="W123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>-670</v>
       </c>
       <c r="X123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>-707</v>
       </c>
       <c r="Y123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>-724</v>
       </c>
       <c r="Z123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>1559</v>
       </c>
       <c r="AA123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>1395</v>
       </c>
       <c r="AB123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>1231</v>
       </c>
       <c r="AC123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>1047</v>
       </c>
       <c r="AD123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>883</v>
       </c>
       <c r="AE123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>719</v>
       </c>
       <c r="AF123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>560</v>
       </c>
       <c r="AG123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>401</v>
       </c>
       <c r="AH123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>22</v>
       </c>
       <c r="AI123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>0</v>
       </c>
       <c r="AJ123" s="47">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>0</v>
       </c>
       <c r="AK123" s="91">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>0</v>
       </c>
     </row>
@@ -26928,123 +27101,123 @@
         <v>#N/A</v>
       </c>
       <c r="H124" s="41" t="e">
-        <f t="shared" ref="H124:AK124" si="34">H123-H119</f>
+        <f t="shared" ref="H124:AK124" si="35">H123-H119</f>
         <v>#N/A</v>
       </c>
       <c r="I124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="J124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="K124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="L124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="M124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="N124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="O124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="P124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="Q124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="R124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="S124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="T124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="U124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="V124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="W124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="X124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="Y124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="Z124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="AA124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="AB124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="AC124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="AD124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="AE124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="AF124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="AG124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="AH124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="AI124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="AJ124" s="41" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
       <c r="AK124" s="42" t="e">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>#N/A</v>
       </c>
     </row>
@@ -27452,8 +27625,9 @@
       <c r="F134" s="55" t="s">
         <v>99</v>
       </c>
-      <c r="G134" s="56" t="e">
-        <v>#N/A</v>
+      <c r="G134" s="56">
+        <f>691</f>
+        <v>691</v>
       </c>
       <c r="H134" s="57" t="e">
         <v>#N/A</v>
@@ -27550,8 +27724,8 @@
       <c r="F135" s="55" t="s">
         <v>100</v>
       </c>
-      <c r="G135" s="56" t="e">
-        <v>#N/A</v>
+      <c r="G135" s="56">
+        <v>669</v>
       </c>
       <c r="H135" s="57" t="e">
         <v>#N/A</v>
@@ -28335,127 +28509,127 @@
         <v>105</v>
       </c>
       <c r="G143" s="46">
-        <f t="shared" ref="G143:AK143" si="35">G79</f>
+        <f t="shared" ref="G143:AK143" si="36">G79</f>
         <v>399</v>
       </c>
       <c r="H143" s="47">
-        <f t="shared" si="35"/>
+        <f>H79</f>
         <v>412</v>
       </c>
       <c r="I143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>425</v>
       </c>
       <c r="J143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>438</v>
       </c>
       <c r="K143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>451</v>
       </c>
       <c r="L143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>464</v>
       </c>
       <c r="M143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>477</v>
       </c>
       <c r="N143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>490</v>
       </c>
       <c r="O143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>503</v>
       </c>
       <c r="P143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>516</v>
       </c>
       <c r="Q143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>529</v>
       </c>
       <c r="R143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>542</v>
       </c>
       <c r="S143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>555</v>
       </c>
       <c r="T143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>568</v>
       </c>
       <c r="U143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>581</v>
       </c>
       <c r="V143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>594</v>
       </c>
       <c r="W143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>607</v>
       </c>
       <c r="X143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>620</v>
       </c>
       <c r="Y143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>633</v>
       </c>
       <c r="Z143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>646</v>
       </c>
       <c r="AA143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>659</v>
       </c>
       <c r="AB143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>672</v>
       </c>
       <c r="AC143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>685</v>
       </c>
       <c r="AD143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>698</v>
       </c>
       <c r="AE143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>711</v>
       </c>
       <c r="AF143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>724</v>
       </c>
       <c r="AG143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>737</v>
       </c>
       <c r="AH143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>750</v>
       </c>
       <c r="AI143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>0</v>
       </c>
       <c r="AJ143" s="47">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>0</v>
       </c>
       <c r="AK143" s="91">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>0</v>
       </c>
     </row>
@@ -28468,138 +28642,141 @@
         <v>#N/A</v>
       </c>
       <c r="H144" s="41" t="e">
-        <f t="shared" ref="H144:AK144" si="36">H143-H139</f>
+        <f>H143-H139</f>
         <v>#N/A</v>
       </c>
       <c r="I144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" ref="H144:AK144" si="37">I143-I139</f>
         <v>#N/A</v>
       </c>
       <c r="J144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="K144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="L144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="M144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="N144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="O144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="P144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="Q144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="R144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="S144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="T144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="U144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="V144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="W144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="X144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="Y144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="Z144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="AA144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="AB144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="AC144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="AD144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="AE144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="AF144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="AG144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="AH144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="AI144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="AJ144" s="41" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
       <c r="AK144" s="42" t="e">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>#N/A</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="A2:A15"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B4:B8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:B14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C4:C8"/>
-    <mergeCell ref="C10:C14"/>
+    <mergeCell ref="A16:A58"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="C62:C72"/>
+    <mergeCell ref="D71:D72"/>
+    <mergeCell ref="D24:D29"/>
+    <mergeCell ref="D42:D45"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="C42:C47"/>
     <mergeCell ref="A80:A81"/>
     <mergeCell ref="C16:C17"/>
     <mergeCell ref="D16:D17"/>
@@ -28616,19 +28793,16 @@
     <mergeCell ref="B37:B47"/>
     <mergeCell ref="B16:B31"/>
     <mergeCell ref="A59:A79"/>
-    <mergeCell ref="A16:A58"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="C62:C72"/>
-    <mergeCell ref="D71:D72"/>
-    <mergeCell ref="D24:D29"/>
-    <mergeCell ref="D42:D45"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="C42:C47"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A2:A15"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="B4:B8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:B14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C4:C8"/>
+    <mergeCell ref="C10:C14"/>
   </mergeCells>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
* * * * * 【2025/09/17 定例会】 改     実際は2025/9/20に実施
０．計画表のバグ修正

　今回はなし

１．各自の立替分の精算
　　＊メイン口座には下記収入15万円があったが、先月より6万円減った。
 			東北電力配当金  	 1
 			全労済東１      	 4
			ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 	 9
 			普通預金利息　　	 1
　　　　従って、今月のメイン口座の支出は21万円前後ということになる。

　　＊共通口座は先月より40万円減った。
　　　月平均30万円程度で減少する想定に対してやや多いが、現金立替分に下記変動項目があったためである。
　　　　　(1)保険料
　　　　　(2)生活費
　　　　　　　　・小遣い振込			 	 7
　　　　　　　　・現金立替分				16			＊含む	ダンス教室回数券				6.4
　　　　　　　　　　　　　　　　　　　　　　　　　　　　　		8月帰省時のSUICA払いの引落分	1.6
　　　　　　　　　　　　　　　　　　　　　　　　　　　　　		南川町内会プレミアム商品券		2.0
　　　　　　　　・その他カード引落分		 ?
　　　　　(3)イベント費
　　　　　		・なし

２．収支の確認
　　＊メイン口座は想定通り。
　　　 ただ楽天カード費4000円がここから引落されることを修正するはずが、行っていない。
　　＊今年度の共通口座はあと残額の661万円使えるが、支出は640万円以内に抑えたい。
　　　　→　月平均30万円で減少すると6か月後の年度末には残金460万円位になるが、
　　　　　　これには、リフォームの400万円，国内旅行（秋の金華山，雅章旅行）30万円を含むので計画ぎりぎりである。
　　　　　　イベント費についてはよく計画値を意識して使う必要がある。

３．メイン口座と共通口座のバランス確認
　　＊特になし

４．計画（ライフプラン.xlsx）の修正
　　＊特になし
</commit_message>
<xml_diff>
--- a/ライフプラン_猪飼.xlsx
+++ b/ライフプラン_猪飼.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC_USER\Documents\LocalLifeplanRepo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD020057-C120-4738-AC61-C472E1FB74AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C402420C-5A87-41EF-A48B-3351A5A0D2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{934FA03D-99BD-49E0-BFEC-291BD79F4879}"/>
   </bookViews>
@@ -107,19 +107,7 @@
       </text>
     </comment>
     <comment ref="G12" authorId="1" shapeId="0" xr:uid="{A75EC272-0EA6-45F5-A5BD-BD752B3901E3}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="MS P ゴシック"/>
-            <family val="3"/>
-            <charset val="128"/>
-          </rPr>
-          <t>便座</t>
-        </r>
-      </text>
+      <text/>
     </comment>
     <comment ref="H12" authorId="1" shapeId="0" xr:uid="{B9A45C49-D949-4109-B5F8-D413C4BCB125}">
       <text>
@@ -877,6 +865,26 @@
         </r>
       </text>
     </comment>
+    <comment ref="G116" authorId="0" shapeId="0" xr:uid="{B56A3F48-96A8-4986-A566-5802F97A6C98}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>kaz
+ 東北電力配当金  + 1
+ 全労済東１      + 4
+ ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 + 9
+ 普通預金利息　　+ 1
+nao</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="F126" authorId="0" shapeId="0" xr:uid="{9D0EDA07-5D89-456F-A52C-3AAD29C57E72}">
       <text>
         <r>
@@ -1009,6 +1017,22 @@
           </rPr>
           <t>kazへ返済 -7 (墓参：1、飯山出雲&amp;鮎：1.2、実家修理：1.6，ﾋﾞｭｰ：1。衣笠浜寿司：1.2、他：1)
 naoへ返済 -2.5（飯山出雲；2，森永：0.2， 町内祭:0.3）</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G136" authorId="0" shapeId="0" xr:uid="{BF817CDE-6E07-46B8-AC4D-02248735669C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>kazへ返済 -6.5 (南川商品券：1、医療費：2、ﾋﾞｭｰ：1、食代など：2.5)
+naoへ返済 -9（ﾀﾞﾝｽ：6.4，南川商品券：1、新潟SUICA費：1.6）</t>
         </r>
       </text>
     </comment>
@@ -6500,7 +6524,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>1118</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -9952,7 +9976,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>630</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -13403,7 +13427,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>1748</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>#N/A</c:v>
@@ -21300,7 +21324,7 @@
         <v>0</v>
       </c>
       <c r="G60" s="69">
-        <f t="shared" ref="F60:AH60" si="9">SUM(G59:G59)</f>
+        <f t="shared" ref="G60:AH60" si="9">SUM(G59:G59)</f>
         <v>824</v>
       </c>
       <c r="H60" s="69">
@@ -23259,7 +23283,7 @@
         <v>0</v>
       </c>
       <c r="G78" s="35">
-        <f t="shared" ref="F78:AH78" si="15">G60-G77</f>
+        <f t="shared" ref="G78:AH78" si="15">G60-G77</f>
         <v>-23</v>
       </c>
       <c r="H78" s="35">
@@ -24593,9 +24617,9 @@
       <c r="F96" s="55" t="s">
         <v>101</v>
       </c>
-      <c r="G96" s="56" t="e">
+      <c r="G96" s="56">
         <f t="shared" ref="G96:AK96" si="25">G116+G136</f>
-        <v>#N/A</v>
+        <v>1748</v>
       </c>
       <c r="H96" s="57" t="e">
         <f t="shared" si="25"/>
@@ -26282,8 +26306,8 @@
       <c r="F116" s="55" t="s">
         <v>101</v>
       </c>
-      <c r="G116" s="56" t="e">
-        <v>#N/A</v>
+      <c r="G116" s="56">
+        <v>1118</v>
       </c>
       <c r="H116" s="57" t="e">
         <v>#N/A</v>
@@ -27823,8 +27847,8 @@
       <c r="F136" s="55" t="s">
         <v>101</v>
       </c>
-      <c r="G136" s="56" t="e">
-        <v>#N/A</v>
+      <c r="G136" s="56">
+        <v>630</v>
       </c>
       <c r="H136" s="57" t="e">
         <v>#N/A</v>
@@ -28647,7 +28671,7 @@
         <v>#N/A</v>
       </c>
       <c r="I144" s="41" t="e">
-        <f t="shared" ref="H144:AK144" si="37">I143-I139</f>
+        <f t="shared" ref="I144:AK144" si="37">I143-I139</f>
         <v>#N/A</v>
       </c>
       <c r="J144" s="41" t="e">
@@ -28807,7 +28831,8 @@
   </mergeCells>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
* * 【2026/4/17 定例会】 改     実際は2026/4/30に実施
０．計画表のバグ修正

　今回はなし

１．各自の立替分の精算
　　＊メイン口座は収入71万円、支出53万円で収支は18万円の黒字になった。
　　　　ただ下記の計画フ実行のため年度初めの預金額が計画値より700万円程多めになっている。
　　　　	・共通口座に2026年分の振込み		561
　　　　	・りそな口座からのリフォーム代補填		100

　　　　　<収入>  71万円
                     国民厚生年金		45
		     パナ年金		12
		     ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金	 9
		     全労済		 4
		     配当金(住友重機)	 1

　　　　　<支出>  53万円
		     マンション管理費	 5
	   	     横浜市固定資産税	 4
	 	     光熱費		 3
		     保険料（ｱｸｻ，ｱﾌﾗｯｸ）	 1
		     小遣い		 7
		     パナ健康保険料	33

　　＊共通口座は今月も先月より26万円減った。平均30万円/月としたほぼ想定通りの支出である。

２．収支の確認
　　＊メイン口座は、今月は収入が多く、18万円の黒字になった。
　　＊年度初めの共通口座は、2016/4/17時点で一旦残金をクリアしてメイン口座からの振込561万円でスタートすべきだが、402万円残っている。
　　　これは上述のように約500万円を見込んだリフォームと、そのために補填するはずだったりそな銀行からの100万円振込を行っていないためである。
　　　　従って、2026年度移行ののイベント計画を見直す必要がある。

３．メイン口座と共通口座のバランス確認
　　＊1年通じた実績で、共通口座の巣出は平均30万円/月でよいと考える。つまり、小遣いも現状のままで妥当であろう。
　　
４．計画（ライフプラン.xlsx）の修正
　　＊上述のようにイベント計画の見直しが必要だが、今回は行っていない。
</commit_message>
<xml_diff>
--- a/ライフプラン_猪飼.xlsx
+++ b/ライフプラン_猪飼.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC_USER\Documents\LocalLifeplanRepo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68EE31E3-AF7A-4C45-9F50-3E90B0B5FF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D78FD0F-695B-4BE8-AC0E-FAC951B15219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="-960" windowWidth="24240" windowHeight="17520" activeTab="1" xr2:uid="{934FA03D-99BD-49E0-BFEC-291BD79F4879}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{934FA03D-99BD-49E0-BFEC-291BD79F4879}"/>
   </bookViews>
   <sheets>
     <sheet name="マネーフロー" sheetId="1" r:id="rId1"/>
     <sheet name="ライフプラン" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -901,6 +902,27 @@
         </r>
       </text>
     </comment>
+    <comment ref="H113" authorId="0" shapeId="0" xr:uid="{B537E54B-069E-4CDE-B3C9-13F66680B0DF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>kaz
+ 国民厚生年金　　　　+45
+ パナ年金　　　  　　+12
+ ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 　 + 9
+ 全労済　　　　 　　 + 4
+ 配当金(住友重機) 　 + 1
+ パナ健康保険料　   -33</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="G114" authorId="0" shapeId="0" xr:uid="{10DA67DA-68D6-4278-954A-276F536F8BA2}">
       <text>
         <r>
@@ -1180,6 +1202,22 @@
 Nao国民健康保険料残金　24
 kazへ返済 -5 (検診､抜歯他)
 naoへ返済 -2（出雲,歯科,黄金柑）</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H133" authorId="0" shapeId="0" xr:uid="{58B7ECF0-45C0-49AB-A615-046CB3F22129}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>kazへ返済 -4.7 (医療費：1.3、ビューカード：0.6、瀬戸神社:0.2、外食：0.2，他：2.4)
+naoへ返済 -6.0（カイロ：0.7，医療費：0.6，ダンス：6.4，ランドリー：0.3，前借【服飾代】：-1.8）</t>
         </r>
       </text>
     </comment>
@@ -4818,10 +4856,8 @@
             <c:v>メイン口座＿1月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -5059,10 +5095,8 @@
             <c:v>メイン口座＿2月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -5300,10 +5334,8 @@
             <c:v>メイン口座＿3月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -5541,10 +5573,8 @@
             <c:v>メイン口座＿4月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -5676,7 +5706,7 @@
                   <c:v>1301</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>#N/A</c:v>
+                  <c:v>1289</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>#N/A</c:v>
@@ -5782,10 +5812,8 @@
             <c:v>メイン口座＿5月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -6023,12 +6051,8 @@
             <c:v>メイン口座＿6月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -6270,12 +6294,8 @@
             <c:v>メイン口座＿7月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -6517,12 +6537,8 @@
             <c:v>メイン口座＿8月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -6764,12 +6780,8 @@
             <c:v>メイン口座＿9月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -7011,12 +7023,8 @@
             <c:v>メイン口座＿10月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -7258,12 +7266,8 @@
             <c:v>メイン口座＿11月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -7505,13 +7509,8 @@
             <c:v>メイン口座＿12月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="80000"/>
-                  <a:lumOff val="20000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -8274,10 +8273,8 @@
             <c:v>共通口座＿1月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -8515,10 +8512,8 @@
             <c:v>共通口座＿2月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -8756,10 +8751,8 @@
             <c:v>共通口座＿3月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -8997,10 +8990,8 @@
             <c:v>共通口座＿4月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -9132,7 +9123,7 @@
                   <c:v>812</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>#N/A</c:v>
+                  <c:v>402</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>#N/A</c:v>
@@ -9238,10 +9229,8 @@
             <c:v>共通口座＿5月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -9722,12 +9711,8 @@
             <c:v>共通口座＿7月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -9969,12 +9954,8 @@
             <c:v>共通口座＿8月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -10216,12 +10197,8 @@
             <c:v>共通口座＿9月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -10463,12 +10440,8 @@
             <c:v>共通口座＿10月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -10710,12 +10683,8 @@
             <c:v>共通口座＿11月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -10957,13 +10926,8 @@
             <c:v>共通口座＿12月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="80000"/>
-                  <a:lumOff val="20000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -12207,10 +12171,8 @@
             <c:v>総合＿3月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -12448,10 +12410,8 @@
             <c:v>総合＿4月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -12583,7 +12543,7 @@
                   <c:v>2113</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>#N/A</c:v>
+                  <c:v>1691</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>#N/A</c:v>
@@ -12689,10 +12649,8 @@
             <c:v>総合＿5月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -13173,12 +13131,8 @@
             <c:v>総合＿7月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -13420,12 +13374,8 @@
             <c:v>総合＿8月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -13667,12 +13617,8 @@
             <c:v>総合＿9月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -13914,12 +13860,8 @@
             <c:v>総合＿10月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -14161,12 +14103,8 @@
             <c:v>総合＿11月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -14408,13 +14346,8 @@
             <c:v>総合＿12月実績</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="80000"/>
-                  <a:lumOff val="20000"/>
-                </a:schemeClr>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -24848,9 +24781,9 @@
         <f t="shared" ref="G93:AK93" si="20">G113+G133</f>
         <v>2113</v>
       </c>
-      <c r="H93" s="57" t="e">
+      <c r="H93" s="57">
         <f t="shared" si="20"/>
-        <v>#N/A</v>
+        <v>1691</v>
       </c>
       <c r="I93" s="57" t="e">
         <f t="shared" si="20"/>
@@ -26692,8 +26625,8 @@
         <f>1701-400</f>
         <v>1301</v>
       </c>
-      <c r="H113" s="57" t="e">
-        <v>#N/A</v>
+      <c r="H113" s="57">
+        <v>1289</v>
       </c>
       <c r="I113" s="57" t="e">
         <v>#N/A</v>
@@ -28231,8 +28164,8 @@
         <f>388+24+400</f>
         <v>812</v>
       </c>
-      <c r="H133" s="57" t="e">
-        <v>#N/A</v>
+      <c r="H133" s="57">
+        <v>402</v>
       </c>
       <c r="I133" s="57" t="e">
         <v>#N/A</v>

</xml_diff>

<commit_message>
* * * 【2026/4717 定例会】 改     実際は2026/8/03に実施
　　この時点で、naoの小遣い口座からの共通口座への返却均は未払い（後日行うとのこと）

　以下省略
</commit_message>
<xml_diff>
--- a/ライフプラン_猪飼.xlsx
+++ b/ライフプラン_猪飼.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC_USER\Documents\LocalLifeplanRepo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783CA1FD-CB8E-4283-A107-621649B536BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE379F5E-949F-4EB9-8F46-DDAF21B132AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{934FA03D-99BD-49E0-BFEC-291BD79F4879}"/>
   </bookViews>
@@ -59,6 +59,32 @@
         </r>
       </text>
     </comment>
+    <comment ref="J6" authorId="0" shapeId="0" xr:uid="{E69F89B2-0434-41FB-A33B-3D28CD80AB17}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>PC_USER:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="H10" authorId="0" shapeId="0" xr:uid="{004E8166-C187-48BE-ACF1-58DC27A96611}">
       <text>
         <r>
@@ -70,7 +96,8 @@
             <family val="3"/>
             <charset val="128"/>
           </rPr>
-          <t>日本一周クルーズ</t>
+          <t>202606：奈良　8　
+日本一周クルーズ</t>
         </r>
       </text>
     </comment>
@@ -884,32 +911,6 @@
         </r>
       </text>
     </comment>
-    <comment ref="M110" authorId="0" shapeId="0" xr:uid="{810AE1A6-2695-4C15-9097-542FE06A2684}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="MS P ゴシック"/>
-            <family val="3"/>
-            <charset val="128"/>
-          </rPr>
-          <t>PC_USER:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="MS P ゴシック"/>
-            <family val="3"/>
-            <charset val="128"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="G113" authorId="0" shapeId="0" xr:uid="{23DA8E04-2475-49BD-AD45-69212BFA74D0}">
       <text>
         <r>
@@ -1011,12 +1012,11 @@
             <family val="3"/>
             <charset val="128"/>
           </rPr>
-          <t xml:space="preserve">kaz
+          <t>kaz
  国民厚生年金　　　　+45
  パナ年金　　　  　　+12
  ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 　 + 9
- 明治安田生命　 　　 + 2
- </t>
+ 明治安田生命　 　　 + 2</t>
         </r>
       </text>
     </comment>
@@ -1036,6 +1036,26 @@
  全労済東１      + 4
  ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 + 9
 nao</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H116" authorId="0" shapeId="0" xr:uid="{178F64E5-DC06-436B-8FD7-0383E78406F2}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t xml:space="preserve">kaz
+ パナ年金　　　  　　+ 6
+ ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 　 + 9
+ 全労済　　　　 　　 + 5
+ 株配当（東北電力）　+ 1
+</t>
         </r>
       </text>
     </comment>
@@ -1361,6 +1381,22 @@
           </rPr>
           <t>kazへ返済 -4 (新潟_網戸&amp;小嶋屋：1.1、医療費：1.4、ﾋﾞｭｰ：1。他)
 naoへ返済 -2.5（出雲；3，森永：0.3， 交通費返却：-0.7）</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H136" authorId="0" shapeId="0" xr:uid="{46C8C73A-BE64-4065-83AA-C5C36B0A63D0}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>kazへ返済 -2.8 (医療費：1.2、ビューカード：0.3，瀬戸神社：0.2 外食：0.2，他：0.9)
+naoへ返済 2.3（森永：0.4，カイロ：0.7，医療費：0.3，ダンス：0.0，全神社：2.9，nao返却：6.6，他：0.2）</t>
         </r>
       </text>
     </comment>
@@ -6525,7 +6561,7 @@
                   <c:v>1076</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>#N/A</c:v>
+                  <c:v>1064</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>#N/A</c:v>
@@ -9942,7 +9978,7 @@
                   <c:v>691</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>#N/A</c:v>
+                  <c:v>322</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>#N/A</c:v>
@@ -13362,7 +13398,7 @@
                   <c:v>1767</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>#N/A</c:v>
+                  <c:v>1386</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>#N/A</c:v>
@@ -25262,9 +25298,9 @@
         <f t="shared" ref="G96:AK96" si="23">G116+G136</f>
         <v>1767</v>
       </c>
-      <c r="H96" s="57" t="e">
+      <c r="H96" s="57">
         <f t="shared" si="23"/>
-        <v>#N/A</v>
+        <v>1386</v>
       </c>
       <c r="I96" s="57" t="e">
         <f t="shared" si="23"/>
@@ -27079,8 +27115,8 @@
       <c r="G116" s="56">
         <v>1076</v>
       </c>
-      <c r="H116" s="57" t="e">
-        <v>#N/A</v>
+      <c r="H116" s="57">
+        <v>1064</v>
       </c>
       <c r="I116" s="57" t="e">
         <v>#N/A</v>
@@ -28619,8 +28655,8 @@
         <f>691</f>
         <v>691</v>
       </c>
-      <c r="H136" s="57" t="e">
-        <v>#N/A</v>
+      <c r="H136" s="57">
+        <v>322</v>
       </c>
       <c r="I136" s="57" t="e">
         <v>#N/A</v>

</xml_diff>

<commit_message>
* * * * 【2026/08/17 定例会】 改     実際は2026/9/02に実施
　　昨年からの実績見直しをした。

　　(1)メイン口座は、年度末では200万円の赤字見込み。公共料金値上げのせいか？

　　　　　＊2026年度は4/17で残金1289万円，8/17で残金1120万円である。
　　　　　　2026/4にnao保険料33万円の支出があったがこれを除くと月平均では
　　　　　　［1120ー（1289-33）]/4＝-34万円/月の減少である。
　　　　　＊年度末ではさらに34*8＝272万円減少するので、残金は848万円程度
　　　　　　　になる見込みである。計画値の495万円を353万円上回っているが、
　　　　　　　これは2026年度の共通口座への561万円払込みが未実施のためであり、
　　　　　　　むしろ、353-561＝-208万円の赤字見込みと考えなければならない。
　　　　　　　　イベント費を削減して、2026年度の払込みを行うべきか要検討！

　　(2)共通口座は、ほぼ想定通り。日常生活費を重視して、イベント費を抑えるべきか？
　　　　　　
　　　　　＊2026年度は4/17で残金402万円，8/17で残金288万円である。
　　　　　　 月平均では、［288ー402]/4＝-28.5万円/月の減少である。
　　　　　＊年度末ではさらに28.5*8＝228万円減少するので、残金は60万円程度
　　　　　　　になる見込みである。計画値の０万円を60万円上回っているが、
　　　　　　　リフォーム未実施で浮いた500万円の、メイン口座からの561万円払込み
　　　　　　　未実施のためで、計画には合っている。
          医療費がかかった割に検討は、旅行を抑えたからかもしれない。
　　　　　 ＊共通口座への振込金は、計画では＋イベント費で計算しているが、
　　　　　　　実績からは、28.5*12＋イベント費＝ 342＋イベント費程度にしたいところ。
　　　　　　　

　以下省略
</commit_message>
<xml_diff>
--- a/ライフプラン_猪飼.xlsx
+++ b/ライフプラン_猪飼.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC_USER\Documents\LocalLifeplanRepo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE379F5E-949F-4EB9-8F46-DDAF21B132AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABAA6CD7-45DC-448E-866B-C6CFA5CBDA06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{934FA03D-99BD-49E0-BFEC-291BD79F4879}"/>
   </bookViews>
@@ -911,6 +911,32 @@
         </r>
       </text>
     </comment>
+    <comment ref="N110" authorId="0" shapeId="0" xr:uid="{D651B64B-A804-4E0F-B522-BFD2BF745BFD}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>PC_USER:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="G113" authorId="0" shapeId="0" xr:uid="{23DA8E04-2475-49BD-AD45-69212BFA74D0}">
       <text>
         <r>
@@ -1075,6 +1101,35 @@
  パナ年金　　　  +12　
  ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 + 9
 nao</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H117" authorId="0" shapeId="0" xr:uid="{602A088E-FE0F-4413-ADF6-80CCD6C93EC9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>kaz
+ 国民厚生年金　　　　+46
+ パナ年金　　　  　　+12
+ ﾌﾟﾙﾃﾞﾝｼｬﾙ保険金 　 + 9</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
         </r>
       </text>
     </comment>
@@ -1413,6 +1468,23 @@
           </rPr>
           <t>kazへ返済 -7 (墓参：1、飯山出雲&amp;鮎：1.2、実家修理：1.6，ﾋﾞｭｰ：1。衣笠浜寿司：1.2、他：1)
 naoへ返済 -2.5（飯山出雲；2，森永：0.2， 町内祭:0.3）</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H137" authorId="0" shapeId="0" xr:uid="{7537FAF8-1843-41AD-9AF8-31F355B90CBC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>kazへ返済 85396 -8.5 (医療費：1.0、ビューカード：0.3，ｺｰﾄﾞﾚｽｸﾘｰﾅｰ:5.0、タクシー：0.1、映画：0.1、外食：0.2，他：1.8)
+naoへ返済 34867 -3.5（森永：0.3，カイロ：0.7，医療費：0.0，ダンス：0.0，出雲大社：1.2，nao返却：-0.3，分踊り飯：0.6，他：1.0)
+ ＊ nao大腸検査 2.2，先月の奈良宿泊費の引落 2.1</t>
         </r>
       </text>
     </comment>
@@ -6804,7 +6876,7 @@
                   <c:v>1124</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>#N/A</c:v>
+                  <c:v>1120</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>#N/A</c:v>
@@ -10221,7 +10293,7 @@
                   <c:v>669</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>#N/A</c:v>
+                  <c:v>288</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>#N/A</c:v>
@@ -13641,7 +13713,7 @@
                   <c:v>1793</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>#N/A</c:v>
+                  <c:v>1408</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>#N/A</c:v>
@@ -25427,9 +25499,9 @@
         <f t="shared" ref="G97:AK97" si="24">G117+G137</f>
         <v>1793</v>
       </c>
-      <c r="H97" s="57" t="e">
+      <c r="H97" s="57">
         <f t="shared" si="24"/>
-        <v>#N/A</v>
+        <v>1408</v>
       </c>
       <c r="I97" s="57" t="e">
         <f t="shared" si="24"/>
@@ -27213,8 +27285,8 @@
       <c r="G117" s="56">
         <v>1124</v>
       </c>
-      <c r="H117" s="57" t="e">
-        <v>#N/A</v>
+      <c r="H117" s="57">
+        <v>1120</v>
       </c>
       <c r="I117" s="57" t="e">
         <v>#N/A</v>
@@ -28753,8 +28825,8 @@
       <c r="G137" s="56">
         <v>669</v>
       </c>
-      <c r="H137" s="57" t="e">
-        <v>#N/A</v>
+      <c r="H137" s="57">
+        <v>288</v>
       </c>
       <c r="I137" s="57" t="e">
         <v>#N/A</v>

</xml_diff>